<commit_message>
feat(evaluation): switch dense workflow to bge-m3
Make the rerun and evaluation path use bge-m3 as the canonical dense model and refresh related notebooks and query artifacts for the current 10K run.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/evaluation/potential_queries/queries_type_5.xlsx
+++ b/data/evaluation/potential_queries/queries_type_5.xlsx
@@ -482,7 +482,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>["no-nbim-ade1c8f19caf6496bf7f28535570cd3e96c97894", "no-nbim-159d40231ae5455d48893546feb071a44ace7ad5", "no-nbim-78befac8721edc5e793fba267238907ba8213f0f", "no-nbim-e3d7a1d6b9e538503945fda52329836ef4c5e12a", "no-nbim-b5ffaebe157f355ce2317383256437b3f007e6b3", "no-nbim-a0a964a7a911acc13fa5a3da83840bd2704ded49", "no-nbim-796013e4261b5a4a88a6c5853ec7083785d96d7f", "no-nbim-c2a31abfe03f36837644ad3332432c0f121e992d", "no-nbim-6963aa70f8bc1065afa55044309c539e200e76fe", "no-nbim-1c325cae92a99ff434adeb885f254e6cdce2fb23", "no-nbim-5da646e195992ea00de285f439331c0313fd765e", "no-nbim-5e181bca7ed78f522d666a1e7bf3d9acfd61dfb0", "no-nbim-234b01471c8df5c244116df53bea7aa3cd6d6d3a", "no-nbim-2ee9948ed42f3eeb4e9ecfd4a64e715b8d92e4c2", "no-nbim-b5491e4ce61db8e2a06ef8efba2634a6f3b29472", "no-nbim-e868d59916cdce206dce8dd9a87e96447aba87e5", "no-nbim-804c2ea28eb68db241f29249a13827e8290d6ad3", "no-nbim-95b9121e72ba3a5bf5841f46b8f1ac17e68d9a9f", "no-nbim-7e192c6f47e3f9d20f6db580a2a0e68855ebbfc1", "no-nbim-889194d9d394477fb4eb10ac19ad56122d55863f", "no-nbim-e2eb51a6760d2825ccd2fa5567274fb95a10ea49", "no-nbim-621da685abf98b1e2255bbde8a3a214bf5fc7d25", "no-nbim-d1d8f5584368072877a1e642ae39c598554b30e9", "no-nbim-fcb700a37c3d71193720c6e3ab0edef59ee64b3d", "no-nbim-b82fc7b10e36cc391e0ccfa0afe55d219fede3fd", "no-nbim-e1a42a8ae233c9144f4d0ca36cc2ffbda8109965", "no-nbim-1beff25f934cee1598161e40b471b52123df54c9", "no-nbim-8f2d54f562811096efc0f8fcd94da387d4065213", "no-nbim-9a5dde38aba3dc077cba72e92bc55a9048d9e065", "no-nbim-81b92a5bf60c13bc18d5e3057e0b6506082e0ecd", "no-nbim-2fd2ea3833ec746e47c74cd4ee9e7d6a425ab7d1", "no-nbim-0efbf06b116806667c55652c6da9050471bda47f", "no-nbim-51b762e0d8ce521b776099612039ebada5dd4977", "no-nbim-c86847f5dbe7dd574ff5f1d69d63f4bb116df62d", "no-nbim-303cbb54a28d4f62fb1e7816842943069cc90842", "no-nbim-9b85dab6c6175df3506bc0960955b0ba384469b6", "no-nbim-7cea9eb3485e897f3718760d5ebd4a89717aea13", "no-nbim-38f9e430e2eb92c832fb872620a363b83bf6f1be", "no-nbim-be943779c692b45c2c3cd3255151263f69a2479e", "no-nbim-730e90a05b69ca08afe4b0000712ce8fb50c5552", "no-nbim-c78a34b47f6f3c85ead2bccd7c1e3e7503801a95", "no-nbim-eb10adc337c95028446d35769d0b6df3c1caf788", "no-nbim-88fccaa43a9727ef731ebe0a68975cebde766a8e", "no-nbim-63a600f743bfe956b9df2af24a7b32125648d180", "no-nbim-b2140bf41caf38f52b626624e29eded4bada394a", "no-nbim-350f5d64493c6e6db84cc98cc2678fd69b9f3f40", "no-nbim-67c789be187a8f7a184e97c9b86c62747ea63a6f", "no-nbim-cafaac304fdba58e3473b57822848a7653887134", "no-nbim-74f3598b9975a10d1f8ecc8859f5702f2a7ab84d", "no-nbim-6e58011b6fb22245db2ec396f115fa7b05f43a8d", "no-nbim-fe57f3867628df5490b8de79359e8b9440f7b108", "no-nbim-1bab50d2c7a294a7323a6dcf2f497f709118abb9", "no-nbim-3b7a452e42023cd81364af5810d88a6191bdb7dd", "no-nbim-dd5ab3dc28c26fcb513dff359d17ce515eea3183", "no-nbim-f0342c9dc21d149138c14beb429b3d00306b312a", "no-nbim-2c4c36430e841be3249b50bfcd4854d75c0bd0e9", "no-nbim-ef7cd2460d64f11f4a0f76798a4357d9c1391b54", "no-nbim-f3ca280a749f3cc4b0733ee9724f28f663f70322", "no-nbim-1e7f2a407934bd09858653996f98358104db95c6", "no-nbim-c42fff5759835bb3d9cb75e3d8ba077b996e4e6a", "no-nbim-ee71258415a706a211f380dc2cc8feb057f028a2", "no-nbim-87924e102df77fa23c073a33bcd066d620a9f07f", "no-nbim-330707a269a23eaa4ed0a1f704c24ac0bbfb503c", "no-nbim-90d90f9c85972361be5367497f2fd9d660e66958", "no-nbim-ccc5b5ecb4e97e2c6e7ec458ab090a64fff700db", "no-nbim-c2c14c0a811b0eed77d6f2d3e0dacf3c31b34122", "no-nbim-11dbe7cd30f588dbf142d6a8bf05e01c8dbfdc3d", "no-nbim-d61e9a8b13306b88a4215e055ec034f3486719d7", "no-nbim-3d3dd0659fdbd1c75694a2da105a6e99ca2febf6", "no-nbim-82dde6bd6b9b4874adb6ab584b3c202acb5e5ae3", "no-nbim-ddc88247fe7b3458f51144a5dfd07db27781aa37", "no-nbim-d2c81029debad5d682d8f5c809f3b41c1b97ed85", "no-nbim-ca86b11d6a04fe6dff6519092f4c2d431a9ffaa6", "no-nbim-6fff0d33812ca525821ac126b668c157cb2dadb3", "no-nbim-2fb09d703cbae64bae53096f662168f8e6559fb0", "no-nbim-de11858b95048a91dd053593b48ab67238cfe34d", "no-nbim-1506cdc8b73168848c19cb8cf3444e6cfcadd742", "no-nbim-73bdf485c77b97920d6cb22d7cd2dbb8230862a5", "no-nbim-b4630a55772a9fc1cb03763261dae20a6558d7e3", "no-nbim-7cf8abeaa6a12c913eb35207ebefc504440be719", "no-nbim-66c31ef33d29e1b522c88ce223960c4caccabbce", "no-nbim-a5f6f61ebfb565a60edf8057889e366f65341225", "no-nbim-65ecf76f6ac314cf50a43772e53b53f39b31faf2", "no-nbim-bf2d032b20742e96ae44babaa466c3cdadd78663", "no-nbim-3da207f65df004979818399e2527af8488030177", "no-nbim-c31d91f4b3e5c4b12a04b5fa7bf67b8f17f9881c", "no-nbim-6263fbd15decf3fa94e6144b5d081e041c0e986c", "no-nbim-3a5ef37a435633c40917e8b687af37e372b3ebbe", "no-nbim-a47fb56985532a7a7bce4d3eca88be7fa2a18ec4", "no-nbim-b08d2577f248c8b1d39b08435dbbd0e9afa59fa8", "no-nbim-fb6018b447bbc40c3a5c32c51cecc1731940166c", "no-nbim-9a30ee913632364d8454d44366d64b2260e27973", "no-nbim-0caa5c5762286eab920dfcce0e402d821197e406", "no-nbim-431a88d91a93b175def555e40b34651101fde85c", "no-nbim-5b72c3bc1fb4744407162a2c0bc07ce62ff5e662", "no-nbim-5e3c08a84f6bf86f34f125c7ff0d15aca7571765", "no-nbim-d8ba644cdb60202fdefa29ec5b52977f9660d6ef", "no-nbim-bd2c52cc245ac8e55b0e575283682c74d3f87516", "no-nbim-f90e0e562feba37217f6ca6e81dd3f0d7f76736b", "no-nbim-b8bee78b0805cd0c5b1555f60284d7b73e9e496b", "no-nbim-b90d5cd1d396053868a7b9e020d58f7754912ad5", "no-nbim-050c2b2b26073cafdaf765f52ae7172fc2480cc9"]</t>
+          <t>["no-nbim-159d40231ae5455d48893546feb071a44ace7ad5", "no-nbim-a0a964a7a911acc13fa5a3da83840bd2704ded49", "no-nbim-c2c14c0a811b0eed77d6f2d3e0dacf3c31b34122", "no-nbim-050c2b2b26073cafdaf765f52ae7172fc2480cc9", "no-nbim-bf2d032b20742e96ae44babaa466c3cdadd78663", "no-nbim-6e58011b6fb22245db2ec396f115fa7b05f43a8d", "no-nbim-c86847f5dbe7dd574ff5f1d69d63f4bb116df62d", "no-nbim-fcb700a37c3d71193720c6e3ab0edef59ee64b3d", "no-nbim-9b85dab6c6175df3506bc0960955b0ba384469b6", "no-nbim-5e3c08a84f6bf86f34f125c7ff0d15aca7571765", "no-nbim-3b7a452e42023cd81364af5810d88a6191bdb7dd", "no-nbim-1beff25f934cee1598161e40b471b52123df54c9", "no-nbim-fb6018b447bbc40c3a5c32c51cecc1731940166c", "no-nbim-b8bee78b0805cd0c5b1555f60284d7b73e9e496b", "no-nbim-234b01471c8df5c244116df53bea7aa3cd6d6d3a", "no-nbim-7cea9eb3485e897f3718760d5ebd4a89717aea13", "no-nbim-5da646e195992ea00de285f439331c0313fd765e", "no-nbim-c42fff5759835bb3d9cb75e3d8ba077b996e4e6a", "no-nbim-2fb09d703cbae64bae53096f662168f8e6559fb0", "no-nbim-66c31ef33d29e1b522c88ce223960c4caccabbce", "no-nbim-d8ba644cdb60202fdefa29ec5b52977f9660d6ef", "no-nbim-621da685abf98b1e2255bbde8a3a214bf5fc7d25", "no-nbim-67c789be187a8f7a184e97c9b86c62747ea63a6f", "no-nbim-cafaac304fdba58e3473b57822848a7653887134", "no-nbim-74f3598b9975a10d1f8ecc8859f5702f2a7ab84d", "no-nbim-78befac8721edc5e793fba267238907ba8213f0f", "no-nbim-b90d5cd1d396053868a7b9e020d58f7754912ad5", "no-nbim-d1d8f5584368072877a1e642ae39c598554b30e9", "no-nbim-be943779c692b45c2c3cd3255151263f69a2479e", "no-nbim-d2c81029debad5d682d8f5c809f3b41c1b97ed85", "no-nbim-ddc88247fe7b3458f51144a5dfd07db27781aa37", "no-nbim-3da207f65df004979818399e2527af8488030177", "no-nbim-1c325cae92a99ff434adeb885f254e6cdce2fb23", "no-nbim-38f9e430e2eb92c832fb872620a363b83bf6f1be", "no-nbim-51b762e0d8ce521b776099612039ebada5dd4977", "no-nbim-7e192c6f47e3f9d20f6db580a2a0e68855ebbfc1", "no-nbim-c31d91f4b3e5c4b12a04b5fa7bf67b8f17f9881c", "no-nbim-f0342c9dc21d149138c14beb429b3d00306b312a", "no-nbim-b82fc7b10e36cc391e0ccfa0afe55d219fede3fd", "no-nbim-9a30ee913632364d8454d44366d64b2260e27973", "no-nbim-11dbe7cd30f588dbf142d6a8bf05e01c8dbfdc3d", "no-nbim-1e7f2a407934bd09858653996f98358104db95c6", "no-nbim-b2140bf41caf38f52b626624e29eded4bada394a", "no-nbim-2fd2ea3833ec746e47c74cd4ee9e7d6a425ab7d1", "no-nbim-de11858b95048a91dd053593b48ab67238cfe34d", "no-nbim-eb10adc337c95028446d35769d0b6df3c1caf788", "no-nbim-fe57f3867628df5490b8de79359e8b9440f7b108", "no-nbim-9a5dde38aba3dc077cba72e92bc55a9048d9e065", "no-nbim-ccc5b5ecb4e97e2c6e7ec458ab090a64fff700db", "no-nbim-7cf8abeaa6a12c913eb35207ebefc504440be719", "no-nbim-82dde6bd6b9b4874adb6ab584b3c202acb5e5ae3", "no-nbim-c2a31abfe03f36837644ad3332432c0f121e992d", "no-nbim-d61e9a8b13306b88a4215e055ec034f3486719d7", "no-nbim-2c4c36430e841be3249b50bfcd4854d75c0bd0e9", "no-nbim-a47fb56985532a7a7bce4d3eca88be7fa2a18ec4", "no-nbim-804c2ea28eb68db241f29249a13827e8290d6ad3", "no-nbim-b4630a55772a9fc1cb03763261dae20a6558d7e3", "no-nbim-95b9121e72ba3a5bf5841f46b8f1ac17e68d9a9f", "no-nbim-0caa5c5762286eab920dfcce0e402d821197e406", "no-nbim-889194d9d394477fb4eb10ac19ad56122d55863f", "no-nbim-a5f6f61ebfb565a60edf8057889e366f65341225", "no-nbim-e868d59916cdce206dce8dd9a87e96447aba87e5", "no-nbim-8f2d54f562811096efc0f8fcd94da387d4065213", "no-nbim-6263fbd15decf3fa94e6144b5d081e041c0e986c", "no-nbim-e1a42a8ae233c9144f4d0ca36cc2ffbda8109965", "no-nbim-ee71258415a706a211f380dc2cc8feb057f028a2", "no-nbim-730e90a05b69ca08afe4b0000712ce8fb50c5552", "no-nbim-90d90f9c85972361be5367497f2fd9d660e66958", "no-nbim-ade1c8f19caf6496bf7f28535570cd3e96c97894", "no-nbim-b5ffaebe157f355ce2317383256437b3f007e6b3", "no-nbim-88fccaa43a9727ef731ebe0a68975cebde766a8e", "no-nbim-b5491e4ce61db8e2a06ef8efba2634a6f3b29472", "no-nbim-3d3dd0659fdbd1c75694a2da105a6e99ca2febf6", "no-nbim-3a5ef37a435633c40917e8b687af37e372b3ebbe", "no-nbim-1bab50d2c7a294a7323a6dcf2f497f709118abb9", "no-nbim-330707a269a23eaa4ed0a1f704c24ac0bbfb503c", "no-nbim-81b92a5bf60c13bc18d5e3057e0b6506082e0ecd", "no-nbim-87924e102df77fa23c073a33bcd066d620a9f07f", "no-nbim-e2eb51a6760d2825ccd2fa5567274fb95a10ea49", "no-nbim-6fff0d33812ca525821ac126b668c157cb2dadb3", "no-nbim-bd2c52cc245ac8e55b0e575283682c74d3f87516", "no-nbim-ef7cd2460d64f11f4a0f76798a4357d9c1391b54", "no-nbim-5e181bca7ed78f522d666a1e7bf3d9acfd61dfb0", "no-nbim-f3ca280a749f3cc4b0733ee9724f28f663f70322", "no-nbim-6963aa70f8bc1065afa55044309c539e200e76fe", "no-nbim-73bdf485c77b97920d6cb22d7cd2dbb8230862a5", "no-nbim-1506cdc8b73168848c19cb8cf3444e6cfcadd742", "no-nbim-dd5ab3dc28c26fcb513dff359d17ce515eea3183", "no-nbim-5b72c3bc1fb4744407162a2c0bc07ce62ff5e662", "no-nbim-0efbf06b116806667c55652c6da9050471bda47f", "no-nbim-c78a34b47f6f3c85ead2bccd7c1e3e7503801a95", "no-nbim-b08d2577f248c8b1d39b08435dbbd0e9afa59fa8", "no-nbim-2ee9948ed42f3eeb4e9ecfd4a64e715b8d92e4c2", "no-nbim-303cbb54a28d4f62fb1e7816842943069cc90842", "no-nbim-431a88d91a93b175def555e40b34651101fde85c", "no-nbim-796013e4261b5a4a88a6c5853ec7083785d96d7f", "no-nbim-350f5d64493c6e6db84cc98cc2678fd69b9f3f40", "no-nbim-f90e0e562feba37217f6ca6e81dd3f0d7f76736b", "no-nbim-63a600f743bfe956b9df2af24a7b32125648d180", "no-nbim-65ecf76f6ac314cf50a43772e53b53f39b31faf2", "no-nbim-ca86b11d6a04fe6dff6519092f4c2d431a9ffaa6", "no-nbim-e3d7a1d6b9e538503945fda52329836ef4c5e12a"]</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -508,7 +508,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>["no-nbim-22dbccdd1ec9dc3906e03a969e8d627d7191131e", "no-nbim-b104ce18553fbe819c6b58f396e363a83d0a542b", "no-nbim-26ba35c37300f5b4b4ad08c1ae78ee3e30477407", "no-nbim-2a102e5081bd08f02c886165624afd09b9402c91", "no-nbim-2f22bf95fbd286459d21d3a36d86836cae210e7c", "no-nbim-1d57b64f6e2b1a6bf4dcfa41de4d20a5ddbcbb40", "no-nbim-ab5fd345b710299175d213291641ce41bacb07eb", "no-nbim-5466ea0bda729a14afd913c74d8e828088a40f1e", "no-nbim-61ecf6cb9f765959641d84c2246eed03f56a8221", "no-nbim-6561452c9c7d18c5c9346826cafb296efa6ef870", "no-nbim-959a358e862195219eccf494de61be926aad83cd", "no-nbim-a6d2f9208bd63599fe6ee5f6ceb95d5cf78714c3", "no-nbim-c2ed7f83fc5d3b1a4edeea7a9a8034822afb2a34", "no-nbim-dc47e4fa68ee842ea8c4ed5e3c827a407708807c", "no-nbim-fdced820a94adfa9ea230fa71ddba574451f44e3", "no-nbim-5a3555db431f6f83cff8ea12547b3dd09be10cef", "no-nbim-05ec714f89832f32ce8f548d2092b5f1f520416e", "no-nbim-0100b85d41846a9ad64492d85e8d32f24f3a8cff", "no-nbim-5b32993d1bda680d678a2134f7e0ebb6c266b44f", "no-nbim-edaf568a7f4b312cdc989209ab49dd027119e943", "no-nbim-2a0e7196bf1eb9f75141f7a7966c071ea4d9d04c", "no-nbim-4fe9c4a9be5f445f8b76202b54ba2b2dc97fdc2a", "no-nbim-4ab546495e328586ce62a448ddc9a7ecbf3144b2", "no-nbim-bdbaaa9d9608812b7ccb5d16dcd1d8f8fa5b6a35", "no-nbim-12344a507f0d838885b3bf90021b8dc35ebce1ae", "no-nbim-33eba4515ab82121e82a40ccc3466a4efb77af51", "no-nbim-f6a1951203dba6598dc41cda5bb5f662e10f9482", "no-nbim-ca708c792fa6ae116ee00248928f8a439fe82808", "no-nbim-d5329925f044f7056c89a2423fb4574b23e6aaaa", "no-nbim-afdadf16b5956e6bac58b6e3834f3133fc696157", "no-nbim-f87f7c03c8f12e8cc59f88f02e91804d37033f5d", "no-nbim-8f926fe8ee4463bff3415f1acfc632e814a32e99", "no-nbim-11266744ed30d8426eeccb0c682262e88166173d", "no-nbim-6327fc13fb7c282ed37934f5e802617089895aad", "no-nbim-bcfab2235a6ce045967d03878aa82e1ad6a6c75a", "no-nbim-e7bb771e88cb2b69307144abc41013dd096d3830", "no-nbim-5eb049e9cc3f95a6a0042ae9cc667f4bf805eaa1", "no-nbim-86ae0c9e8f44fae6fe61f44e3eb3ea30bb3163f8", "no-nbim-8794bbf6d88310777801fdcebf08cf627feaf55f", "no-nbim-278e05831dedf955a8a9e75c921791bcb45dd5d5", "no-nbim-2611455c26159c7d3a6a7cb0c59199fff5d8ca7b", "no-nbim-201f2e6430c0d3a6aa44312d2611b4afeb20ec77", "no-nbim-6a22a03a2f43a40e1648b882ad89b7a093753bb9", "no-nbim-7573bdef05f827a5d6f2f0b07fa8b01a3ca5157b", "no-nbim-db72171e5901f891e2d41f3a2588d0e711e6c70c", "no-nbim-8f9928ce8009512b01f2593992a242542df70a47", "no-nbim-9117947ec52d822f4268d41f8fcace342204d196", "no-nbim-5677917a8644c486e109d0e27bb955f7e426605e", "no-nbim-e8c1d2d2ba57c18e384a2b74ea798879ac355156", "no-nbim-6bc98ba17ebbbcbbc2a559b4287f21b60437e7de", "no-nbim-dddedccd90848bb5118def1417688f4198fdae49", "no-nbim-cbf26a242626ff71250698f606aa40a99ce98cdf", "no-nbim-6afe49ebe81bac22f816c5af86f116383a190206", "no-nbim-7dcdaf1558218b9dfcc1a94964d942345f340c21", "no-nbim-9ad7de15726f2ed086dbb294db3145b9b08f244e", "no-nbim-5d8526722c0646a7d80ef9c30888141c1b4b253a", "no-nbim-6acbfa0b96d9fe0dd2bade51e867cf001ac9b9c5", "no-nbim-6c4e0af83f6cbc36b450e638fb11509fd6da3f9e", "no-nbim-a15bf394c3d6e77a21be77eabb282e16393ce2b8", "no-nbim-1ef091b0443360ab5801a1004cce4f7da9088a4d", "no-nbim-e1bc2bb6c458435aff9f022f5857bf1f8db73330", "no-nbim-af7062a6f52602169c8e8fe3c31ed751801f1538", "no-nbim-dc83820109e9b5a60c4511dd826d584c9ad6921e", "no-nbim-005da79574c3c9e30892461a3dec7d8cbaae5f83", "no-nbim-27b65ab6a993e4882242ae029883fe2cb2270bcb", "no-nbim-02b8f21a8eca3d22bb737832f9430b449d76cc33", "no-nbim-229885536d10bd94f471a501c864b09a1c387864", "no-nbim-63a6606e136c735f43d2d0a89a39b6c0750b6b6f", "no-nbim-8a31b742cc0efbcc969b48f6dd2484d78c1b2a6f", "no-nbim-b28446444957073c9fb900caf46c65b233ad65e7", "no-nbim-b7a418f8029bd3ecf81c1501760576f58bf750dc", "no-nbim-c68b4f4c80add95f91cd2108c25b4bbc7a810472", "no-nbim-7e342695b81dae90e24dbaf344624adf3b1c7d8b", "no-nbim-bc6751a6b538c594ac2d487205b5f3741d1dde9f"]</t>
+          <t>["no-nbim-e7bb771e88cb2b69307144abc41013dd096d3830", "no-nbim-4ab546495e328586ce62a448ddc9a7ecbf3144b2", "no-nbim-8a31b742cc0efbcc969b48f6dd2484d78c1b2a6f", "no-nbim-5eb049e9cc3f95a6a0042ae9cc667f4bf805eaa1", "no-nbim-dddedccd90848bb5118def1417688f4198fdae49", "no-nbim-fdced820a94adfa9ea230fa71ddba574451f44e3", "no-nbim-b28446444957073c9fb900caf46c65b233ad65e7", "no-nbim-63a6606e136c735f43d2d0a89a39b6c0750b6b6f", "no-nbim-bcfab2235a6ce045967d03878aa82e1ad6a6c75a", "no-nbim-5677917a8644c486e109d0e27bb955f7e426605e", "no-nbim-ca708c792fa6ae116ee00248928f8a439fe82808", "no-nbim-278e05831dedf955a8a9e75c921791bcb45dd5d5", "no-nbim-e8c1d2d2ba57c18e384a2b74ea798879ac355156", "no-nbim-33eba4515ab82121e82a40ccc3466a4efb77af51", "no-nbim-5466ea0bda729a14afd913c74d8e828088a40f1e", "no-nbim-61ecf6cb9f765959641d84c2246eed03f56a8221", "no-nbim-6c4e0af83f6cbc36b450e638fb11509fd6da3f9e", "no-nbim-af7062a6f52602169c8e8fe3c31ed751801f1538", "no-nbim-afdadf16b5956e6bac58b6e3834f3133fc696157", "no-nbim-26ba35c37300f5b4b4ad08c1ae78ee3e30477407", "no-nbim-8f926fe8ee4463bff3415f1acfc632e814a32e99", "no-nbim-6327fc13fb7c282ed37934f5e802617089895aad", "no-nbim-c68b4f4c80add95f91cd2108c25b4bbc7a810472", "no-nbim-05ec714f89832f32ce8f548d2092b5f1f520416e", "no-nbim-a15bf394c3d6e77a21be77eabb282e16393ce2b8", "no-nbim-02b8f21a8eca3d22bb737832f9430b449d76cc33", "no-nbim-5a3555db431f6f83cff8ea12547b3dd09be10cef", "no-nbim-229885536d10bd94f471a501c864b09a1c387864", "no-nbim-2a102e5081bd08f02c886165624afd09b9402c91", "no-nbim-7dcdaf1558218b9dfcc1a94964d942345f340c21", "no-nbim-2611455c26159c7d3a6a7cb0c59199fff5d8ca7b", "no-nbim-9117947ec52d822f4268d41f8fcace342204d196", "no-nbim-dc83820109e9b5a60c4511dd826d584c9ad6921e", "no-nbim-ab5fd345b710299175d213291641ce41bacb07eb", "no-nbim-959a358e862195219eccf494de61be926aad83cd", "no-nbim-5b32993d1bda680d678a2134f7e0ebb6c266b44f", "no-nbim-201f2e6430c0d3a6aa44312d2611b4afeb20ec77", "no-nbim-005da79574c3c9e30892461a3dec7d8cbaae5f83", "no-nbim-1d57b64f6e2b1a6bf4dcfa41de4d20a5ddbcbb40", "no-nbim-2f22bf95fbd286459d21d3a36d86836cae210e7c", "no-nbim-6561452c9c7d18c5c9346826cafb296efa6ef870", "no-nbim-86ae0c9e8f44fae6fe61f44e3eb3ea30bb3163f8", "no-nbim-c2ed7f83fc5d3b1a4edeea7a9a8034822afb2a34", "no-nbim-11266744ed30d8426eeccb0c682262e88166173d", "no-nbim-7573bdef05f827a5d6f2f0b07fa8b01a3ca5157b", "no-nbim-6bc98ba17ebbbcbbc2a559b4287f21b60437e7de", "no-nbim-db72171e5901f891e2d41f3a2588d0e711e6c70c", "no-nbim-bdbaaa9d9608812b7ccb5d16dcd1d8f8fa5b6a35", "no-nbim-27b65ab6a993e4882242ae029883fe2cb2270bcb", "no-nbim-edaf568a7f4b312cdc989209ab49dd027119e943", "no-nbim-6afe49ebe81bac22f816c5af86f116383a190206", "no-nbim-2a0e7196bf1eb9f75141f7a7966c071ea4d9d04c", "no-nbim-f6a1951203dba6598dc41cda5bb5f662e10f9482", "no-nbim-d5329925f044f7056c89a2423fb4574b23e6aaaa", "no-nbim-6acbfa0b96d9fe0dd2bade51e867cf001ac9b9c5", "no-nbim-bc6751a6b538c594ac2d487205b5f3741d1dde9f", "no-nbim-e1bc2bb6c458435aff9f022f5857bf1f8db73330", "no-nbim-f87f7c03c8f12e8cc59f88f02e91804d37033f5d", "no-nbim-9ad7de15726f2ed086dbb294db3145b9b08f244e", "no-nbim-12344a507f0d838885b3bf90021b8dc35ebce1ae", "no-nbim-a6d2f9208bd63599fe6ee5f6ceb95d5cf78714c3", "no-nbim-0100b85d41846a9ad64492d85e8d32f24f3a8cff", "no-nbim-4fe9c4a9be5f445f8b76202b54ba2b2dc97fdc2a", "no-nbim-6a22a03a2f43a40e1648b882ad89b7a093753bb9", "no-nbim-8794bbf6d88310777801fdcebf08cf627feaf55f", "no-nbim-8f9928ce8009512b01f2593992a242542df70a47", "no-nbim-b104ce18553fbe819c6b58f396e363a83d0a542b", "no-nbim-dc47e4fa68ee842ea8c4ed5e3c827a407708807c", "no-nbim-5d8526722c0646a7d80ef9c30888141c1b4b253a", "no-nbim-22dbccdd1ec9dc3906e03a969e8d627d7191131e", "no-nbim-b7a418f8029bd3ecf81c1501760576f58bf750dc", "no-nbim-1ef091b0443360ab5801a1004cce4f7da9088a4d", "no-nbim-cbf26a242626ff71250698f606aa40a99ce98cdf", "no-nbim-7e342695b81dae90e24dbaf344624adf3b1c7d8b"]</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -534,7 +534,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>["no-nbim-5c635e68e383978a47ab7bafc22f9d28c9288a33", "no-nbim-f430c99747a03fe42d8e3c9cf9f131d671d05bae", "no-nbim-933bf1a048f19afff587b8f3fe9375dfcaa551d5", "no-nbim-a39e3e17efae78653ebc6f18f43cf5876bd579c8", "no-nbim-9b67daaa68170e4e0d062611524388c4f50cf6d0", "no-nbim-27e266679e472b7398a521ae7e90bd4eb2d89fae", "no-nbim-4c74ae7e058db34a0f66a81a1bae1d0a4672bd85", "no-nbim-17f03d2aae44b125d58101632805b1ba7684f08b", "no-nbim-7eff739c096a334de7917fad1cd343f10c75efd1", "no-nbim-a58711efd2e9dea7e2828408a314796aeef2371a", "no-nbim-8daf88ae08516af38cad1dfb31d681261815ae1c", "no-nbim-47b380051fe0efa2c3dc813113143ac6e9f7f7c7", "no-nbim-f146d0a97cedd17ce886ec021f05710ff624407e", "no-nbim-e1cb830e318ec203d12a08733c214e96aa8cc8d2", "no-nbim-bf30a020d61c2c128d70affdefb94af85de958a0", "no-nbim-a6d16dfc5337dcb8d2066164664c1e96a216f3e8", "no-nbim-cd90b207e7291cb38fed76363f72f3556f428eab", "no-nbim-b61ac814d2d98675b854754244e9df81b71810f3", "no-nbim-df88e10477c03b4cfc530cd0e5d1744f82234f92", "no-nbim-fed4d6f48b3a7ed22b9afdfe44c6fcd96e2335cf", "no-nbim-e91d18e17726149eb306dd0ec76f33c82c67cca2", "no-nbim-9179cb29a74c77457b7926509f71570700241abd", "no-nbim-9c5f1a218b8c699151371a0c7c6a4557e870d290", "no-nbim-aa365c737fc1726ae8dbbf47b6bff57df9f9da77", "no-nbim-77c618dff09b05529a99bc6c1595b57acf04a9f0", "no-nbim-f266e2378558850a79abae180517098fac7b1c0e", "no-nbim-7e86f32a4198c21d5152dcf84fcee3a981d3cc5b", "no-nbim-650ab486d26454a1c2adb3d6d75e0114c32985a0", "no-nbim-389934f3b21de026dcf500e1105370a12bca57c4", "no-nbim-2d5ce458433b87cb6ee4ee986ce56e403b92a5f7", "no-nbim-319173469c0162f082412a5ee9daf033f0f66fd3", "no-nbim-087ed013485a52328e21953c5bcaa2ae959273c0", "no-nbim-bc6600ca61a365cbee47ef9c54f4cdaf928afc5a", "no-nbim-dcc8a5e2c8a67d410fc4660fc091acb6008f598d", "no-nbim-3a79509473eca26d9708e932f94d9a9facb719df", "no-nbim-98bd75aa562faffe23b6be94fc87504784694d22", "no-nbim-fa345d47b282601d0193aeb0e0f79cef2063ed19", "no-nbim-bdf8462befc085eb6a000c498853fc807d8a7fa6", "no-nbim-23f5ad6b20e9292a6dcfa879798ecf8e6353d517", "no-nbim-32ea4078520b350f463ef4ed4e87149ada8b0eb3", "no-nbim-945abfe111863feea13471b155985d641863f818", "no-nbim-257d3452879fcb9a6834a271e4ba0b56716d2b20", "no-nbim-ab3776e7d93299c3295f0d5735d51e06bc90dde9", "no-nbim-96074cfb2a61b57dc458cc61a58386298d15d1d0", "no-nbim-6aca56503d808b84a26703e5e1812865bf42e3eb", "no-nbim-c8004d3f978a5e357ccac81c9718769b46381c22", "no-nbim-dd7a550bb001daa16bf3c3a00c69722cd5ae1841", "no-nbim-90fcd7a368f12aa95b37d89f615ee6d6c09175c9", "no-nbim-c940df0fca65dba9934ed92d9c8aa1f8b1bca193", "no-nbim-06fe93e36164bc439b94d80a5f65e9202f8c770d", "no-nbim-b01eb188d5980e0372b747ddf4382c1af0e37942", "no-nbim-16e07ac7e88636eb443afec1d374bfccbdad5bb6", "no-nbim-9ab064602a9bd3434161d01f82b8af8a10c1784d", "no-nbim-b10102e2dbee0dbdf17c806640011ab6f1f7e55b", "no-nbim-ccf8ab4a7acf6db52fec0bf624890d8ffc62ddab", "no-nbim-cc28e7b3d9f55d5a64787dff19abbc8cbea4d1cc", "no-nbim-d7c017411abbacca166746f6b102e84c68fb9d5a", "no-nbim-56e6ae14c2d556435e5939244a4b35dee3de2198", "no-nbim-5410e3ac47aa4d50ebede788626f6595c33f8ffd", "no-nbim-c120318bd4b2320ca4f6b0463d2635ccad90ae67", "no-nbim-5c00bbac742e672d7b6eea6632f7a03816ab74fe", "no-nbim-771479d29387d24b0df80d2d14a179c646c9fb43", "no-nbim-8f7ce6ac619b41f6d3bb3d6a45f3aec733d0b2e5", "no-nbim-15c6cdb4f7be9c7dca8c8fdccbeedbda07e5a3b1", "no-nbim-8f00c04b7f6a7a1c797b3987ccbc96081c829687", "no-nbim-7177a26dfb92b9423d89a02700fc8057f75c51af", "no-nbim-730ac4d166d52502f50e5f7b557309ed835d7f10", "no-nbim-bab628839d6060282fc141bc1e990ce88b271963", "no-nbim-7337ebc7f226ba0b9e979428efe238a6c76700be"]</t>
+          <t>["no-nbim-257d3452879fcb9a6834a271e4ba0b56716d2b20", "no-nbim-c940df0fca65dba9934ed92d9c8aa1f8b1bca193", "no-nbim-a39e3e17efae78653ebc6f18f43cf5876bd579c8", "no-nbim-dd7a550bb001daa16bf3c3a00c69722cd5ae1841", "no-nbim-b61ac814d2d98675b854754244e9df81b71810f3", "no-nbim-bc6600ca61a365cbee47ef9c54f4cdaf928afc5a", "no-nbim-06fe93e36164bc439b94d80a5f65e9202f8c770d", "no-nbim-8f00c04b7f6a7a1c797b3987ccbc96081c829687", "no-nbim-933bf1a048f19afff587b8f3fe9375dfcaa551d5", "no-nbim-319173469c0162f082412a5ee9daf033f0f66fd3", "no-nbim-ab3776e7d93299c3295f0d5735d51e06bc90dde9", "no-nbim-5c00bbac742e672d7b6eea6632f7a03816ab74fe", "no-nbim-9ab064602a9bd3434161d01f82b8af8a10c1784d", "no-nbim-3a79509473eca26d9708e932f94d9a9facb719df", "no-nbim-16e07ac7e88636eb443afec1d374bfccbdad5bb6", "no-nbim-b10102e2dbee0dbdf17c806640011ab6f1f7e55b", "no-nbim-4c74ae7e058db34a0f66a81a1bae1d0a4672bd85", "no-nbim-56e6ae14c2d556435e5939244a4b35dee3de2198", "no-nbim-32ea4078520b350f463ef4ed4e87149ada8b0eb3", "no-nbim-47b380051fe0efa2c3dc813113143ac6e9f7f7c7", "no-nbim-bf30a020d61c2c128d70affdefb94af85de958a0", "no-nbim-f146d0a97cedd17ce886ec021f05710ff624407e", "no-nbim-dcc8a5e2c8a67d410fc4660fc091acb6008f598d", "no-nbim-6aca56503d808b84a26703e5e1812865bf42e3eb", "no-nbim-7177a26dfb92b9423d89a02700fc8057f75c51af", "no-nbim-fed4d6f48b3a7ed22b9afdfe44c6fcd96e2335cf", "no-nbim-b01eb188d5980e0372b747ddf4382c1af0e37942", "no-nbim-945abfe111863feea13471b155985d641863f818", "no-nbim-a58711efd2e9dea7e2828408a314796aeef2371a", "no-nbim-8f7ce6ac619b41f6d3bb3d6a45f3aec733d0b2e5", "no-nbim-5c635e68e383978a47ab7bafc22f9d28c9288a33", "no-nbim-9179cb29a74c77457b7926509f71570700241abd", "no-nbim-aa365c737fc1726ae8dbbf47b6bff57df9f9da77", "no-nbim-a6d16dfc5337dcb8d2066164664c1e96a216f3e8", "no-nbim-bdf8462befc085eb6a000c498853fc807d8a7fa6", "no-nbim-c120318bd4b2320ca4f6b0463d2635ccad90ae67", "no-nbim-5410e3ac47aa4d50ebede788626f6595c33f8ffd", "no-nbim-df88e10477c03b4cfc530cd0e5d1744f82234f92", "no-nbim-e1cb830e318ec203d12a08733c214e96aa8cc8d2", "no-nbim-17f03d2aae44b125d58101632805b1ba7684f08b", "no-nbim-cd90b207e7291cb38fed76363f72f3556f428eab", "no-nbim-15c6cdb4f7be9c7dca8c8fdccbeedbda07e5a3b1", "no-nbim-087ed013485a52328e21953c5bcaa2ae959273c0", "no-nbim-389934f3b21de026dcf500e1105370a12bca57c4", "no-nbim-9c5f1a218b8c699151371a0c7c6a4557e870d290", "no-nbim-c8004d3f978a5e357ccac81c9718769b46381c22", "no-nbim-771479d29387d24b0df80d2d14a179c646c9fb43", "no-nbim-8daf88ae08516af38cad1dfb31d681261815ae1c", "no-nbim-ccf8ab4a7acf6db52fec0bf624890d8ffc62ddab", "no-nbim-98bd75aa562faffe23b6be94fc87504784694d22", "no-nbim-9b67daaa68170e4e0d062611524388c4f50cf6d0", "no-nbim-730ac4d166d52502f50e5f7b557309ed835d7f10", "no-nbim-fa345d47b282601d0193aeb0e0f79cef2063ed19", "no-nbim-90fcd7a368f12aa95b37d89f615ee6d6c09175c9", "no-nbim-f430c99747a03fe42d8e3c9cf9f131d671d05bae", "no-nbim-7eff739c096a334de7917fad1cd343f10c75efd1", "no-nbim-7e86f32a4198c21d5152dcf84fcee3a981d3cc5b", "no-nbim-bab628839d6060282fc141bc1e990ce88b271963", "no-nbim-77c618dff09b05529a99bc6c1595b57acf04a9f0", "no-nbim-27e266679e472b7398a521ae7e90bd4eb2d89fae", "no-nbim-23f5ad6b20e9292a6dcfa879798ecf8e6353d517", "no-nbim-e91d18e17726149eb306dd0ec76f33c82c67cca2", "no-nbim-cc28e7b3d9f55d5a64787dff19abbc8cbea4d1cc", "no-nbim-7337ebc7f226ba0b9e979428efe238a6c76700be", "no-nbim-650ab486d26454a1c2adb3d6d75e0114c32985a0", "no-nbim-2d5ce458433b87cb6ee4ee986ce56e403b92a5f7", "no-nbim-d7c017411abbacca166746f6b102e84c68fb9d5a", "no-nbim-96074cfb2a61b57dc458cc61a58386298d15d1d0", "no-nbim-f266e2378558850a79abae180517098fac7b1c0e"]</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -560,7 +560,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>["isin-RU000A109UL0", "isin-RU000A10CM71", "isin-RU000A1082M3", "isin-RU000A109JX8", "isin-RU000A108UJ6", "isin-RU000A10ASF9", "isin-RU000A10D3R8", "isin-RU000A10BLP1", "isin-RU000A10A0H8", "isin-RU000A1084N7", "isin-RU000A108FG3", "isin-RU000A10AA77", "isin-RU000A10BV89", "isin-RU000A10CAQ0", "isin-RU000A109NM3", "isin-RU000A10DRX8", "isin-RU000A108LL1", "isin-RU000A10A794", "isin-RU000A10AMP1", "isin-RU000A10CR92", "isin-RU000A109KG1", "isin-RU000A10DYZ9", "isin-RU000A10DBH5", "isin-RU000A1085A1", "isin-RU000A10A7A8", "isin-RU000A1097X8", "isin-RU000A10ED70", "isin-RU000A10CM14", "isin-RU000A10DY35", "isin-RU000A10E4F0", "isin-RU000A108405", "isin-RU000A10AYU6", "isin-RU000A1092T7", "isin-RU000A10DTB0", "isin-RU000A10BP46", "isin-RU000A10D4E4", "isin-RU000A10DRV2", "isin-RU000A109783", "isin-RU000A10CM89", "isin-RU000A10BGE5", "isin-RU000A1098U2", "isin-RU000A10ARR6", "isin-RU000A10EAQ6", "isin-RU000A10B2U6", "isin-RU000A108B83", "isin-RU000A107PM2", "isin-RU000A10CSR0", "isin-RU000A10CLZ8", "isin-RU000A10DDG3", "isin-RU000A10DEM9", "isin-RU000A109KK3", "isin-RU000A109AU3", "isin-RU000A10CRA8", "isin-RU000A10CT09", "isin-RU000A10DWP4", "isin-RU000A10C873", "isin-RU000A109MH5", "isin-RU000A10AHP1", "isin-RU000A108WJ2", "isin-RU000A10E7D8", "isin-RU000A109RX1", "isin-RU000A108CE5", "isin-RU000A10BR02"]</t>
+          <t>["isin-RU000A10EAQ6", "isin-RU000A1082M3", "isin-RU000A10ARR6", "isin-RU000A10DRX8", "isin-RU000A10AA77", "isin-RU000A10BR02", "isin-RU000A10AYU6", "isin-RU000A10CM14", "isin-RU000A10CRA8", "isin-RU000A1085A1", "isin-RU000A108LL1", "isin-RU000A10CLZ8", "isin-RU000A10B2U6", "isin-RU000A10DWP4", "isin-RU000A1092T7", "isin-RU000A10DBH5", "isin-RU000A10CR92", "isin-RU000A109783", "isin-RU000A10ED70", "isin-RU000A108B83", "isin-RU000A10A7A8", "isin-RU000A10AMP1", "isin-RU000A10DDG3", "isin-RU000A109RX1", "isin-RU000A1098U2", "isin-RU000A10DY35", "isin-RU000A108405", "isin-RU000A108CE5", "isin-RU000A10C873", "isin-RU000A10CAQ0", "isin-RU000A10AHP1", "isin-RU000A10BV89", "isin-RU000A10DRV2", "isin-RU000A10A0H8", "isin-RU000A109KK3", "isin-RU000A109UL0", "isin-RU000A10E7D8", "isin-RU000A10CM89", "isin-RU000A108UJ6", "isin-RU000A109AU3", "isin-RU000A109MH5", "isin-RU000A10CSR0", "isin-RU000A108FG3", "isin-RU000A10CM71", "isin-RU000A10D3R8", "isin-RU000A10D4E4", "isin-RU000A10DEM9", "isin-RU000A109JX8", "isin-RU000A10A794", "isin-RU000A10ASF9", "isin-RU000A10BLP1", "isin-RU000A1084N7", "isin-RU000A10E4F0", "isin-RU000A107PM2", "isin-RU000A109KG1", "isin-RU000A10DTB0", "isin-RU000A10CT09", "isin-RU000A10BGE5", "isin-RU000A109NM3", "isin-RU000A10BP46", "isin-RU000A1097X8", "isin-RU000A108WJ2", "isin-RU000A10DYZ9"]</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -586,7 +586,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>["isin-RU000A105Y14", "isin-RU000A103NJ2", "isin-RU000A103455", "isin-RU000A103YF7", "isin-RU000A106Y70", "isin-RU000A106T85", "isin-RU000A105PR5", "isin-RU000A1050X7", "isin-RU000A105SZ2", "isin-RU000A105YQ9", "isin-RU000A1029A9", "isin-RU000A106938", "isin-RU000A107EC7", "isin-RU000A105CS1", "isin-RU000A104XW2", "isin-RU000A104WS2", "isin-RU000A105TR7", "isin-RU000A103H25", "isin-RU000A106EV9", "isin-RU000A1021G3", "isin-RU000A1034T9", "isin-RU000A102RU2", "isin-RU000A1035D0", "isin-RU000A103W26", "isin-RU000A104A39", "isin-RU000A104CJ3", "isin-RU000A101RF5", "isin-RU000A1064X8", "isin-RU000A107EW5", "isin-RU000A103YP6", "isin-RU000A106DK4", "isin-RU000A107761", "isin-RU000A102028", "isin-RU000A105BP9", "isin-RU000A103RT2", "isin-RU000A1074F4", "isin-RU000A1028C7", "isin-RU000A102LW1", "isin-RU000A1052T1", "isin-RU000A105YA3", "isin-RU000A103935", "isin-RU000A105GS2", "isin-RU000A105FM7", "isin-RU000A1057A0", "isin-RU000A102TT0", "isin-RU000A103TV4", "isin-RU000A103WB0", "isin-RU000A1032S5", "isin-RU000A105UZ8", "isin-RU000A102B30", "isin-RU000A105CL6", "isin-RU000A1075D6"]</t>
+          <t>["isin-RU000A1052T1", "isin-RU000A105UZ8", "isin-RU000A105Y14", "isin-RU000A1034T9", "isin-RU000A1032S5", "isin-RU000A1064X8", "isin-RU000A102RU2", "isin-RU000A1029A9", "isin-RU000A103W26", "isin-RU000A103YF7", "isin-RU000A104CJ3", "isin-RU000A107761", "isin-RU000A105TR7", "isin-RU000A101RF5", "isin-RU000A1075D6", "isin-RU000A1021G3", "isin-RU000A105YA3", "isin-RU000A104WS2", "isin-RU000A1074F4", "isin-RU000A107EC7", "isin-RU000A1028C7", "isin-RU000A103H25", "isin-RU000A106938", "isin-RU000A105GS2", "isin-RU000A102B30", "isin-RU000A103NJ2", "isin-RU000A103TV4", "isin-RU000A105SZ2", "isin-RU000A102LW1", "isin-RU000A102028", "isin-RU000A106T85", "isin-RU000A105YQ9", "isin-RU000A103455", "isin-RU000A1035D0", "isin-RU000A104A39", "isin-RU000A105BP9", "isin-RU000A103WB0", "isin-RU000A103935", "isin-RU000A102TT0", "isin-RU000A105FM7", "isin-RU000A1050X7", "isin-RU000A106DK4", "isin-RU000A1057A0", "isin-RU000A105CS1", "isin-RU000A103YP6", "isin-RU000A106Y70", "isin-RU000A107EW5", "isin-RU000A103RT2", "isin-RU000A104XW2", "isin-RU000A105PR5", "isin-RU000A105CL6", "isin-RU000A106EV9"]</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -612,7 +612,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>["no-nbim-f2711db3ace6b3923197ccbc5ab07c88ab85de6d", "no-nbim-7c57ff0a0dcc699b19d8ee1c7252d20b2c4080b7", "no-nbim-5db7361e8217c57bad601198eab0ed42cfa2e113", "no-nbim-745f867000cc982938cb62503bf06e54c1b62760", "no-nbim-b1367437f1a6c37c53172b26e1b9beabb7cde073", "no-nbim-8b87af5e57b0a9582792ce732f36732a8e904e98", "no-nbim-7231ea89baba7fe0612495ca66daf4dab0016858", "no-nbim-6a2b199890dda3e61e70663d9d061343ed7f0b44", "no-nbim-b1128c55443c59beacc549745949bba9bc9ca832", "no-nbim-8b6a4bf554175bc617f45779bd74e6b580f48d81", "no-nbim-f7a6fc14e5830607e0d82cc21143bfe98835c1f9", "no-nbim-24243066d8808900aa83aad2fa3f82386391a8be", "no-nbim-29bd28f22abd51b575faac7f3f4f57516df73a0f", "no-nbim-f39839208b0452ed95cd9b2b933e9dba5cd426f6", "no-nbim-18ac276d696774a60180d87f79f22e9ec3e92cd6", "no-nbim-1259ddfa74fe8561a65d5568fecbf8fc7d390ce9", "no-nbim-04d3d652aaec156cefc30392e20e9df135838dc6", "no-nbim-58096145169614c85eefb247eae4f2776439292c", "no-nbim-7280750abc4a0ce7f520542cfbc615b38b125b08", "no-nbim-f27c928d32e25ff14143dfaa155709a3f8af6d73", "no-nbim-c3e7b46c47e084d1f49a6a6f7fdea8afe85f43a0", "no-nbim-e6c0bb13870cf1a430085d1effa48e3c64a0770c", "no-nbim-323e056b6b99094d7b46513044cf7bb6dda21363", "no-nbim-ae8bd900e412a004ca50c48a29483cdbfc6c7382", "no-nbim-00cd9b92225ae348d3a41182debacd7c675fbdba", "no-nbim-e59a37b02764ab08103acda79120d57f92b0e9d8", "no-nbim-0a21f9d92e5d22044b4008330265e0fc3eda14a8", "no-nbim-cdac1d70dc611fe9778008c596cdbac9bc5aae30", "no-nbim-6e3d73ce559ae8dc9cb6f017f468fe2cd5183250", "no-nbim-03f813220194494c6f4378503809964840ae59e5", "no-nbim-e46b432878c7e0d42f4d69b67f27481eb4cb26ca", "no-nbim-8dd4ac8c9a64929fa592eac8ecb635ed02ccc012", "no-nbim-488abc09a736121d7e91a31f8bbc2cd7ba70eda0", "no-nbim-3f8405c26d8a9ee2ba4a4fb3a77175463619c6f9", "no-nbim-378eac5fdd03ceb7ba88e2762ec799972edf7e05", "no-nbim-4c1a5b47ef9e9139d3714247191f7848de77531a", "no-nbim-72808d6520e3a318d0311bfe40018ef29abb3b67", "no-nbim-a98688027ef696057436ac536d2806e08f08ce2a", "no-nbim-6f19cd1f4fad120cd33757084eb0ba0668b2534d", "no-nbim-2aba23c8d3974ea46ccc69e2f91fb8f535351988"]</t>
+          <t>["no-nbim-7c57ff0a0dcc699b19d8ee1c7252d20b2c4080b7", "no-nbim-e59a37b02764ab08103acda79120d57f92b0e9d8", "no-nbim-f2711db3ace6b3923197ccbc5ab07c88ab85de6d", "no-nbim-f39839208b0452ed95cd9b2b933e9dba5cd426f6", "no-nbim-a98688027ef696057436ac536d2806e08f08ce2a", "no-nbim-7280750abc4a0ce7f520542cfbc615b38b125b08", "no-nbim-e46b432878c7e0d42f4d69b67f27481eb4cb26ca", "no-nbim-8b87af5e57b0a9582792ce732f36732a8e904e98", "no-nbim-323e056b6b99094d7b46513044cf7bb6dda21363", "no-nbim-29bd28f22abd51b575faac7f3f4f57516df73a0f", "no-nbim-2aba23c8d3974ea46ccc69e2f91fb8f535351988", "no-nbim-1259ddfa74fe8561a65d5568fecbf8fc7d390ce9", "no-nbim-3f8405c26d8a9ee2ba4a4fb3a77175463619c6f9", "no-nbim-5db7361e8217c57bad601198eab0ed42cfa2e113", "no-nbim-00cd9b92225ae348d3a41182debacd7c675fbdba", "no-nbim-6a2b199890dda3e61e70663d9d061343ed7f0b44", "no-nbim-745f867000cc982938cb62503bf06e54c1b62760", "no-nbim-ae8bd900e412a004ca50c48a29483cdbfc6c7382", "no-nbim-0a21f9d92e5d22044b4008330265e0fc3eda14a8", "no-nbim-6f19cd1f4fad120cd33757084eb0ba0668b2534d", "no-nbim-4c1a5b47ef9e9139d3714247191f7848de77531a", "no-nbim-8b6a4bf554175bc617f45779bd74e6b580f48d81", "no-nbim-24243066d8808900aa83aad2fa3f82386391a8be", "no-nbim-03f813220194494c6f4378503809964840ae59e5", "no-nbim-b1367437f1a6c37c53172b26e1b9beabb7cde073", "no-nbim-58096145169614c85eefb247eae4f2776439292c", "no-nbim-cdac1d70dc611fe9778008c596cdbac9bc5aae30", "no-nbim-f7a6fc14e5830607e0d82cc21143bfe98835c1f9", "no-nbim-378eac5fdd03ceb7ba88e2762ec799972edf7e05", "no-nbim-7231ea89baba7fe0612495ca66daf4dab0016858", "no-nbim-f27c928d32e25ff14143dfaa155709a3f8af6d73", "no-nbim-72808d6520e3a318d0311bfe40018ef29abb3b67", "no-nbim-18ac276d696774a60180d87f79f22e9ec3e92cd6", "no-nbim-c3e7b46c47e084d1f49a6a6f7fdea8afe85f43a0", "no-nbim-e6c0bb13870cf1a430085d1effa48e3c64a0770c", "no-nbim-488abc09a736121d7e91a31f8bbc2cd7ba70eda0", "no-nbim-6e3d73ce559ae8dc9cb6f017f468fe2cd5183250", "no-nbim-b1128c55443c59beacc549745949bba9bc9ca832", "no-nbim-04d3d652aaec156cefc30392e20e9df135838dc6", "no-nbim-8dd4ac8c9a64929fa592eac8ecb635ed02ccc012"]</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>["isin-RU000A10B7N0", "isin-RU000A109F05", "isin-RU000A10ABR0", "isin-RU000A108YZ4", "isin-RU000A109RF8", "isin-RU000A10B4F3", "isin-RU000A10D7Z2", "isin-RU000A10ADR6", "isin-RU000A10BVY2", "isin-RU000A1089A3", "isin-RU000A10ANT1", "isin-RU000A10BQV8", "isin-RU000A108RM6", "isin-RU000A10B2D2", "isin-RU000A10D4S4", "isin-RU000A10BQG9", "isin-RU000A109XN0", "isin-RU000A109L49", "isin-RU000A10EJR5", "isin-RU000A10BYZ3", "isin-RU000A109098", "isin-RU000A1094U1", "isin-RU000A10AHD7", "isin-RU000A109KT4", "isin-RU000A108AC3", "isin-RU000A10CTK3", "isin-RU000A108Q78", "isin-RU000A109S83", "isin-RU000A108ZP2", "isin-RU000A10AHU1", "isin-RU000A10CT74", "isin-RU000A109U06", "isin-RU000A10BQC8", "isin-RU000A109SX9", "isin-RU000A109T41"]</t>
+          <t>["isin-RU000A1089A3", "isin-RU000A108Q78", "isin-RU000A10BQG9", "isin-RU000A109F05", "isin-RU000A10B2D2", "isin-RU000A10B7N0", "isin-RU000A108YZ4", "isin-RU000A10BVY2", "isin-RU000A109098", "isin-RU000A108RM6", "isin-RU000A10AHU1", "isin-RU000A10BQV8", "isin-RU000A109SX9", "isin-RU000A1094U1", "isin-RU000A108AC3", "isin-RU000A10CT74", "isin-RU000A10ABR0", "isin-RU000A109XN0", "isin-RU000A10ADR6", "isin-RU000A10B4F3", "isin-RU000A10BQC8", "isin-RU000A109RF8", "isin-RU000A10BYZ3", "isin-RU000A10AHD7", "isin-RU000A10D7Z2", "isin-RU000A109KT4", "isin-RU000A10CTK3", "isin-RU000A108ZP2", "isin-RU000A109L49", "isin-RU000A10ANT1", "isin-RU000A109T41", "isin-RU000A109S83", "isin-RU000A109U06", "isin-RU000A10D4S4", "isin-RU000A10EJR5"]</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -664,7 +664,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>["us-bis-export-3a54f4c0aa1f1c46015a7bcc75ba79fc322cf53b", "us-bis-export-48d12bddd52d720d8df51e16548342f9e00a422f", "us-bis-export-5b2c46e83495915773d00c93ebb8c29de2c7a2b0", "us-bis-export-7adf27a15c0879d581a15f8e05368dc22d3da6c9", "us-bis-export-67fb9be62a0d9cc537897480269a5c132259bd0e", "us-bis-export-e09801131ff8870f4e4418de5489263669cc9e85", "us-bis-export-e64b37eedd8c2accbaaab47741c503b9fbdab2d9", "us-bis-export-1018bfb459a547dbd2de6f9e35e1c9cf70f2159f", "us-bis-export-15d2dd51273581e9cc181c4346abadee248bcdbb", "us-bis-export-398de17a0513103daeab46b698f17e587d81d6c7", "us-bis-export-addc9eaad7179f57be7289b1ad6cb13813eed376", "us-bis-export-ffa489e53e4322e29ff62bb29116133a2e640b84", "us-bis-export-72f8a753b6ea15f37ea3f8a1fbeb94b6148e5701", "us-bis-export-fd3dd63bbacb452583e792fdc4631bd6cf34d2ed", "us-bis-export-0cddfa861dc5fdbca697069e947d0b39cccf3991", "us-bis-export-fe6986e7a930fd85f4aa91d6707d01d239239716", "us-bis-export-53d825803367590e2ccd23bb0c88d521a0c5d3ea", "us-bis-export-cb0c0836584877297ce648f3c480b2bca54fce27", "us-bis-export-cff61b07488f65cd314c507f72c0aa454b493c97", "us-bis-export-214f003a24cdfb02f6e94cab417f141a4b4f5b0f", "us-bis-export-4f4bcc6e49ae204f24ee26ff9faecf9482754235", "us-bis-export-c651a1aaa4785cd33ebfe7219386c2ba056fd4c4", "us-bis-export-72c7352f384bf6c3db45bd897bc249dc39b77ada", "us-bis-export-da5bffa6186b357e2e12e02d081e3948a7735d32", "us-bis-export-089c4214fc08b24b46a81c4c933bce3cceb2a983", "us-bis-export-b04a4c7e159c56e5262282b71259e77be2fa39a1", "us-bis-export-68f642482c246dc91a331d362cb8b7d8352b1ccb", "us-bis-export-fc20e35cd3e3aa6caf7348933f1573ed792ce600", "us-bis-export-aaebdf3c71a78be66c31dcbe6211d60214de8b61", "us-bis-export-aa0810be7df98690a0af1cf23781eff12cf25c92", "us-bis-export-715a374e32ee019298b1007d7055227517b36c7c", "us-bis-export-80aebefac84569a5fa588ce4e9cfa2d809645f61", "us-bis-export-ff0b6c55f0349af6220392a53dd4e261fe3a2435", "us-bis-export-f69cee8a19aaead98b1717b4a096e87d9ad83625", "us-bis-export-017905e6ca881e90a4e6b614f41816e61ffa48ba"]</t>
+          <t>["us-bis-export-ffa489e53e4322e29ff62bb29116133a2e640b84", "us-bis-export-0cddfa861dc5fdbca697069e947d0b39cccf3991", "us-bis-export-68f642482c246dc91a331d362cb8b7d8352b1ccb", "us-bis-export-53d825803367590e2ccd23bb0c88d521a0c5d3ea", "us-bis-export-214f003a24cdfb02f6e94cab417f141a4b4f5b0f", "us-bis-export-7adf27a15c0879d581a15f8e05368dc22d3da6c9", "us-bis-export-5b2c46e83495915773d00c93ebb8c29de2c7a2b0", "us-bis-export-e64b37eedd8c2accbaaab47741c503b9fbdab2d9", "us-bis-export-fe6986e7a930fd85f4aa91d6707d01d239239716", "us-bis-export-cb0c0836584877297ce648f3c480b2bca54fce27", "us-bis-export-72c7352f384bf6c3db45bd897bc249dc39b77ada", "us-bis-export-1018bfb459a547dbd2de6f9e35e1c9cf70f2159f", "us-bis-export-3a54f4c0aa1f1c46015a7bcc75ba79fc322cf53b", "us-bis-export-aa0810be7df98690a0af1cf23781eff12cf25c92", "us-bis-export-c651a1aaa4785cd33ebfe7219386c2ba056fd4c4", "us-bis-export-ff0b6c55f0349af6220392a53dd4e261fe3a2435", "us-bis-export-fd3dd63bbacb452583e792fdc4631bd6cf34d2ed", "us-bis-export-4f4bcc6e49ae204f24ee26ff9faecf9482754235", "us-bis-export-15d2dd51273581e9cc181c4346abadee248bcdbb", "us-bis-export-aaebdf3c71a78be66c31dcbe6211d60214de8b61", "us-bis-export-f69cee8a19aaead98b1717b4a096e87d9ad83625", "us-bis-export-017905e6ca881e90a4e6b614f41816e61ffa48ba", "us-bis-export-addc9eaad7179f57be7289b1ad6cb13813eed376", "us-bis-export-b04a4c7e159c56e5262282b71259e77be2fa39a1", "us-bis-export-398de17a0513103daeab46b698f17e587d81d6c7", "us-bis-export-80aebefac84569a5fa588ce4e9cfa2d809645f61", "us-bis-export-e09801131ff8870f4e4418de5489263669cc9e85", "us-bis-export-67fb9be62a0d9cc537897480269a5c132259bd0e", "us-bis-export-715a374e32ee019298b1007d7055227517b36c7c", "us-bis-export-fc20e35cd3e3aa6caf7348933f1573ed792ce600", "us-bis-export-da5bffa6186b357e2e12e02d081e3948a7735d32", "us-bis-export-72f8a753b6ea15f37ea3f8a1fbeb94b6148e5701", "us-bis-export-cff61b07488f65cd314c507f72c0aa454b493c97", "us-bis-export-48d12bddd52d720d8df51e16548342f9e00a422f", "us-bis-export-089c4214fc08b24b46a81c4c933bce3cceb2a983"]</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>["isin-MD0000000132", "isin-MD00000001G1", "isin-MD00000001H9", "isin-MD0000000140", "isin-MD00000000R0", "isin-MD00000000P4", "isin-MD0000000173", "isin-MD00000000Z3", "isin-MD0000000199", "isin-MD00000001D8", "isin-MD00000000Y6", "isin-MD00000001A4", "isin-MD00000000V2", "isin-MD00000001K3", "isin-MD0000000157", "isin-MD00000000M1", "isin-MD00000000T6", "isin-MD00000001J5", "isin-MD00000000U4", "isin-MD00000000X8", "isin-MD00000000N9", "isin-MD00000001B2", "isin-MD0000000124", "isin-MD00000001E6", "isin-MD00000000W0", "isin-MD0000000116", "isin-MD00000000S8", "isin-MD00000001C0", "isin-MD0000000108", "isin-MD00000000Q2", "isin-MD00000001F3", "isin-MD0000000165", "isin-MD0000000181"]</t>
+          <t>["isin-MD00000000Y6", "isin-MD00000001A4", "isin-MD0000000173", "isin-MD00000000S8", "isin-MD0000000124", "isin-MD00000000X8", "isin-MD00000001C0", "isin-MD00000001J5", "isin-MD00000000T6", "isin-MD0000000165", "isin-MD0000000157", "isin-MD0000000199", "isin-MD00000001B2", "isin-MD00000000Z3", "isin-MD00000001G1", "isin-MD0000000116", "isin-MD00000000U4", "isin-MD0000000108", "isin-MD0000000132", "isin-MD00000001H9", "isin-MD00000000P4", "isin-MD00000001D8", "isin-MD00000000R0", "isin-MD0000000140", "isin-MD0000000181", "isin-MD00000000N9", "isin-MD00000000M1", "isin-MD00000000W0", "isin-MD00000001E6", "isin-MD00000001K3", "isin-MD00000000Q2", "isin-MD00000000V2", "isin-MD00000001F3"]</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -716,7 +716,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>["us-bis-export-b949a1aced01a5ceac0b4d5a3af1bc2ce495ba98", "us-bis-export-31f361cc0390b229ad15bea91b071dcc5de6dd90", "us-bis-export-a9fc187c0be07e688652ce2cf5f87d7f93bbc19a", "us-bis-export-03a23ae39a5008dd9c442562dabebe478398990c", "us-bis-export-2431f0791bdc64b4ed4a8153303bf5852174987b", "us-bis-export-b26be92e21c8c1d9466e438b753fb8c1253706c5", "us-bis-export-0d60a0eb7d57a2f8f47629f59be30ecdb1931910", "us-bis-export-bf5a966121434970439120344a45d42244cc287e", "us-bis-export-d55836d80b606eb7a271e482b28cec8e7aacff93", "us-bis-export-ffe0df675b44752d79dc997052d0fbfe1e93979f", "us-bis-export-301fd5f060900e2224fa455052547bb1694513de", "us-bis-export-7e189a7e488822a4c1554f0474013861621bce61", "us-bis-export-92748483e3b0f4e0b74b4c4b674aedb71d15ed6f", "us-bis-export-bcd168d2e45968950cdc7f993ea6c2fa4e1119b4", "us-bis-export-3da8479afaffe46a28787d3da8e77ac121c82cbb", "us-bis-export-983c71596a66e17f9f014b74b251fb274dbcfc8c", "us-bis-export-73dc8e9c4cb57e4de4a8fe96d0118eeae00d8617", "us-bis-export-2a4ee3d6809f07c16d71aff66747c090e0bccec8", "us-bis-export-e24e38dfa01950f2b8a80030db095ec0082df0e8", "us-bis-export-31f7d5711f771edc5006c21468c587539af67120", "us-bis-export-4fa60884e751c73b6644ee582fa06fab6f90ffaa", "us-bis-export-940a74de0548faef86a2558abdc06808bdcdd325", "us-bis-export-c6cf3e802d69999e3e468b98de6ae9782a952e2f", "us-bis-export-06bb0a79def0ef22e344fdbd504bfeb1ce0dfe4a", "us-bis-export-815509e0754998f325e7738d9889f1f309ef58af", "us-bis-export-bcf1cd55b6a04526b5fd75dcd526a39f323d9387", "us-bis-export-27d191f5b81119c5f709a3ac40d40c7959f006a6", "us-bis-export-3fb735923314992d912c21e90622d82f347395f9", "us-bis-export-a0ccfd123bf8cc372b9134176df810f1c760ef54", "us-bis-export-88602ee629430a369cb009335d124599cb3f156d", "us-bis-export-6f42780a26246d310b4d0ea598214d4a3e962766", "us-bis-export-44be864c9ad2512a200a2fe7f631e2b08312b19f"]</t>
+          <t>["us-bis-export-d55836d80b606eb7a271e482b28cec8e7aacff93", "us-bis-export-31f7d5711f771edc5006c21468c587539af67120", "us-bis-export-0d60a0eb7d57a2f8f47629f59be30ecdb1931910", "us-bis-export-2431f0791bdc64b4ed4a8153303bf5852174987b", "us-bis-export-88602ee629430a369cb009335d124599cb3f156d", "us-bis-export-815509e0754998f325e7738d9889f1f309ef58af", "us-bis-export-bf5a966121434970439120344a45d42244cc287e", "us-bis-export-31f361cc0390b229ad15bea91b071dcc5de6dd90", "us-bis-export-92748483e3b0f4e0b74b4c4b674aedb71d15ed6f", "us-bis-export-73dc8e9c4cb57e4de4a8fe96d0118eeae00d8617", "us-bis-export-c6cf3e802d69999e3e468b98de6ae9782a952e2f", "us-bis-export-7e189a7e488822a4c1554f0474013861621bce61", "us-bis-export-940a74de0548faef86a2558abdc06808bdcdd325", "us-bis-export-983c71596a66e17f9f014b74b251fb274dbcfc8c", "us-bis-export-27d191f5b81119c5f709a3ac40d40c7959f006a6", "us-bis-export-e24e38dfa01950f2b8a80030db095ec0082df0e8", "us-bis-export-4fa60884e751c73b6644ee582fa06fab6f90ffaa", "us-bis-export-b949a1aced01a5ceac0b4d5a3af1bc2ce495ba98", "us-bis-export-a9fc187c0be07e688652ce2cf5f87d7f93bbc19a", "us-bis-export-b26be92e21c8c1d9466e438b753fb8c1253706c5", "us-bis-export-a0ccfd123bf8cc372b9134176df810f1c760ef54", "us-bis-export-301fd5f060900e2224fa455052547bb1694513de", "us-bis-export-06bb0a79def0ef22e344fdbd504bfeb1ce0dfe4a", "us-bis-export-44be864c9ad2512a200a2fe7f631e2b08312b19f", "us-bis-export-6f42780a26246d310b4d0ea598214d4a3e962766", "us-bis-export-bcd168d2e45968950cdc7f993ea6c2fa4e1119b4", "us-bis-export-03a23ae39a5008dd9c442562dabebe478398990c", "us-bis-export-3da8479afaffe46a28787d3da8e77ac121c82cbb", "us-bis-export-bcf1cd55b6a04526b5fd75dcd526a39f323d9387", "us-bis-export-ffe0df675b44752d79dc997052d0fbfe1e93979f", "us-bis-export-2a4ee3d6809f07c16d71aff66747c090e0bccec8", "us-bis-export-3fb735923314992d912c21e90622d82f347395f9"]</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -742,7 +742,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>["us-bis-export-2b220cadc3050cc042a8f9fa68e0156a8efb2007", "us-bis-export-1cef5f66404333a52a94b912423647c9b75b34f6", "us-bis-export-fa39e47b91c1c90eade87fd8b67a2d7972e96aec", "us-bis-export-c502ecf6d529ee0254d8ac7d265dd1490cf6ab9b", "us-bis-export-a9e84cb9b949de92ebfd16c886b9f605e878f4db", "us-bis-export-b4d96d2f9caa77a03d23b9b4a473f52ab22acb31", "us-bis-export-955fea2f9fb09617dda89b7528c773f14580990d", "us-bis-export-4ce440334e69c64c29963b028b8b97b2c3fa802a", "us-bis-export-a6a1dc9f781c40d887dc717159b449d53525fe74", "us-bis-export-ddcf913041bce9f96b2cc2466b9f02b1bd063c1e", "us-bis-export-51b2e4e85ff629d1c3e456dec6d9f573d6ed6170", "us-bis-export-488c38fe4ce0d8d151804c0c7549084bdafae9cd", "us-bis-export-b9055cb42114695988163440d36f8721c9002869", "us-bis-export-f99313b649d12e4ccae17071aeccfee9b2631eeb", "us-bis-export-415c2bcdf7a09e593791cd9a81972970d66e054b", "us-bis-export-9847035a4242a1c67459f37cb2c06ada021324a4", "us-bis-export-d6ec79f11520eae93b93462fd847b11e1d72bf17", "us-bis-export-e2140c02fdd068e95baf3f050a892b5524004c4f", "us-bis-export-b2bd96ae85c35a3f9751b34c881f017a6eb1f0e0", "us-bis-export-ef1183c391fa262a91b4e73be4fc0cd67b4948fb", "us-bis-export-91789ce0d07d33dddd8b4d5cb9bc9b9db4f74f13", "us-bis-export-7a7db7f27d843f1d169217e393e41d2f0bde84ac", "us-bis-export-80b852d2c75f4cc0ab0acce03004223141a2eeb9", "us-bis-export-5bf8e4ecd7e131917e72b6ef0883929aa373564c", "us-bis-export-8a01baf8766fb7992d3cbe4409af6c640da98ced", "us-bis-export-90bc1c356cd2a51a1a97fe05e282732f8348f015", "us-bis-export-11787cb69f7a602f005bef26ae3349973eb7060b", "us-bis-export-6b106cf13ccb9fd8815bfaa6996016e4fc857ad3", "us-bis-export-72de6bd48d0053431c9dd42bcf09f430b2f99b05", "us-bis-export-f12307bf48e679aad730086ec0b61fa7b69a6284", "us-bis-export-2ac84fa5eb1bdda9761c6023570852144036a326", "us-bis-export-759ffef9195d76d4a25aa9a2e32cf840679ae8a4"]</t>
+          <t>["us-bis-export-ef1183c391fa262a91b4e73be4fc0cd67b4948fb", "us-bis-export-f99313b649d12e4ccae17071aeccfee9b2631eeb", "us-bis-export-ddcf913041bce9f96b2cc2466b9f02b1bd063c1e", "us-bis-export-91789ce0d07d33dddd8b4d5cb9bc9b9db4f74f13", "us-bis-export-6b106cf13ccb9fd8815bfaa6996016e4fc857ad3", "us-bis-export-90bc1c356cd2a51a1a97fe05e282732f8348f015", "us-bis-export-51b2e4e85ff629d1c3e456dec6d9f573d6ed6170", "us-bis-export-b9055cb42114695988163440d36f8721c9002869", "us-bis-export-c502ecf6d529ee0254d8ac7d265dd1490cf6ab9b", "us-bis-export-d6ec79f11520eae93b93462fd847b11e1d72bf17", "us-bis-export-b2bd96ae85c35a3f9751b34c881f017a6eb1f0e0", "us-bis-export-488c38fe4ce0d8d151804c0c7549084bdafae9cd", "us-bis-export-a6a1dc9f781c40d887dc717159b449d53525fe74", "us-bis-export-1cef5f66404333a52a94b912423647c9b75b34f6", "us-bis-export-f12307bf48e679aad730086ec0b61fa7b69a6284", "us-bis-export-759ffef9195d76d4a25aa9a2e32cf840679ae8a4", "us-bis-export-7a7db7f27d843f1d169217e393e41d2f0bde84ac", "us-bis-export-5bf8e4ecd7e131917e72b6ef0883929aa373564c", "us-bis-export-e2140c02fdd068e95baf3f050a892b5524004c4f", "us-bis-export-9847035a4242a1c67459f37cb2c06ada021324a4", "us-bis-export-72de6bd48d0053431c9dd42bcf09f430b2f99b05", "us-bis-export-a9e84cb9b949de92ebfd16c886b9f605e878f4db", "us-bis-export-2b220cadc3050cc042a8f9fa68e0156a8efb2007", "us-bis-export-4ce440334e69c64c29963b028b8b97b2c3fa802a", "us-bis-export-2ac84fa5eb1bdda9761c6023570852144036a326", "us-bis-export-415c2bcdf7a09e593791cd9a81972970d66e054b", "us-bis-export-80b852d2c75f4cc0ab0acce03004223141a2eeb9", "us-bis-export-b4d96d2f9caa77a03d23b9b4a473f52ab22acb31", "us-bis-export-fa39e47b91c1c90eade87fd8b67a2d7972e96aec", "us-bis-export-8a01baf8766fb7992d3cbe4409af6c640da98ced", "us-bis-export-11787cb69f7a602f005bef26ae3349973eb7060b", "us-bis-export-955fea2f9fb09617dda89b7528c773f14580990d"]</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -768,7 +768,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>["isin-RU000A1074E7", "isin-RU000A106VN0", "isin-RU000A103WD6", "isin-RU000A107G63", "isin-RU000A106W49", "isin-RU000A1053W3", "isin-RU000A105BW5", "isin-RU000A105RU5", "isin-RU000A1049M2", "isin-RU000A107DD7", "isin-RU000A107225", "isin-RU000A104C78", "isin-RU000A104UY4", "isin-RU000A103G83", "isin-RU000A105AX5", "isin-RU000A106YD5", "isin-RU000A106ZZ5", "isin-RU000A104BU2", "isin-RU000A103FT7", "isin-RU000A106TJ2", "isin-RU000A102580", "isin-RU000A107PE9", "isin-RU000A105ZF9", "isin-RU000A105VP7", "isin-RU000A1032D7", "isin-RU000A107BD1", "isin-RU000A101PV6", "isin-RU000A104A05", "isin-RU000A104WZ7", "isin-RU000A104V59", "isin-RU000A104W82"]</t>
+          <t>["isin-RU000A103WD6", "isin-RU000A103G83", "isin-RU000A104C78", "isin-RU000A104W82", "isin-RU000A1032D7", "isin-RU000A106W49", "isin-RU000A107PE9", "isin-RU000A102580", "isin-RU000A1053W3", "isin-RU000A107225", "isin-RU000A106VN0", "isin-RU000A105ZF9", "isin-RU000A105BW5", "isin-RU000A107BD1", "isin-RU000A105RU5", "isin-RU000A104V59", "isin-RU000A106ZZ5", "isin-RU000A107DD7", "isin-RU000A106TJ2", "isin-RU000A105AX5", "isin-RU000A104UY4", "isin-RU000A104WZ7", "isin-RU000A103FT7", "isin-RU000A105VP7", "isin-RU000A107G63", "isin-RU000A1074E7", "isin-RU000A1049M2", "isin-RU000A104A05", "isin-RU000A104BU2", "isin-RU000A106YD5", "isin-RU000A101PV6"]</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -794,7 +794,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>["isin-RU000A1057D4", "isin-RU000A106GC4", "isin-RU000A102AB8", "isin-RU000A107LU4", "isin-RU000A106A86", "isin-RU000A106U74", "isin-RU000A1079G1", "isin-RU000A106AK0", "isin-RU000A103604", "isin-RU000A107AZ6", "isin-RU000A101UR4", "isin-RU000A104CK1", "isin-RU000A105EP3", "isin-RU000A102TR4", "isin-RU000A105YB1", "isin-RU000A1061L9", "isin-RU000A109QN4", "isin-RU000A105JG1", "isin-RU000A103RY2", "isin-RU000A1051U1", "isin-RU000A105LS2", "isin-RU000A106HB4", "isin-RU000A107548", "isin-RU000A107E08", "isin-RU000A106XJ4", "isin-RU000A1034J0", "isin-RU000A101RH1", "isin-RU000A106CB5", "isin-RU000A108462", "isin-RU000A104G90", "isin-RU000A1046N6"]</t>
+          <t>["isin-RU000A106A86", "isin-RU000A105YB1", "isin-RU000A1057D4", "isin-RU000A104CK1", "isin-RU000A106AK0", "isin-RU000A107LU4", "isin-RU000A106HB4", "isin-RU000A101RH1", "isin-RU000A106GC4", "isin-RU000A1034J0", "isin-RU000A107AZ6", "isin-RU000A107548", "isin-RU000A105LS2", "isin-RU000A106U74", "isin-RU000A102TR4", "isin-RU000A103RY2", "isin-RU000A103604", "isin-RU000A104G90", "isin-RU000A102AB8", "isin-RU000A1061L9", "isin-RU000A107E08", "isin-RU000A105EP3", "isin-RU000A106XJ4", "isin-RU000A109QN4", "isin-RU000A1079G1", "isin-RU000A1051U1", "isin-RU000A106CB5", "isin-RU000A105JG1", "isin-RU000A101UR4", "isin-RU000A108462", "isin-RU000A1046N6"]</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -820,7 +820,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>["isin-RU000A10B7W1", "isin-RU000A10DMN0", "isin-RU000A10CU30", "isin-RU000A10AZG2", "isin-RU000A10C8H9", "isin-RU000A10B1X2", "isin-RU000A10BWA0", "isin-RU000A1098H9", "isin-RU000A10A7H3", "isin-RU000A10AA02", "isin-RU000A10B0R6", "isin-RU000A10E9V6", "isin-RU000A109KV0", "isin-RU000A109SM2", "isin-RU000A10EL13", "isin-RU000A10A9K3", "isin-RU000A10AGA5", "isin-RU000A108G70", "isin-RU000A109SH2", "isin-RU000A10ECR0", "isin-RU000A10B255", "isin-RU000A108ZQ0", "isin-RU000A107T76", "isin-RU000A10BU72", "isin-RU000A1086N2", "isin-RU000A10BJL4", "isin-RU000A10D665", "isin-RU000A10AYB6", "isin-RU000A10EK63", "isin-RU000A10AHJ4", "isin-RU000A107YT9"]</t>
+          <t>["isin-RU000A10BWA0", "isin-RU000A10BU72", "isin-RU000A10BJL4", "isin-RU000A10AHJ4", "isin-RU000A10CU30", "isin-RU000A10D665", "isin-RU000A1086N2", "isin-RU000A10AYB6", "isin-RU000A10DMN0", "isin-RU000A108G70", "isin-RU000A10B1X2", "isin-RU000A10AZG2", "isin-RU000A10EL13", "isin-RU000A10EK63", "isin-RU000A10A7H3", "isin-RU000A10ECR0", "isin-RU000A109SM2", "isin-RU000A108ZQ0", "isin-RU000A10E9V6", "isin-RU000A107T76", "isin-RU000A10B7W1", "isin-RU000A107YT9", "isin-RU000A10A9K3", "isin-RU000A10B255", "isin-RU000A109SH2", "isin-RU000A10C8H9", "isin-RU000A109KV0", "isin-RU000A10AA02", "isin-RU000A1098H9", "isin-RU000A10B0R6", "isin-RU000A10AGA5"]</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -846,7 +846,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>["us-bis-export-1878696a0dfcc2b4df8fe4c1b4c18ea191d2379a", "us-bis-export-1f6b4cd4b222a77730cdc398d633455b1f54f068", "us-bis-export-a5e2916444556c0a92de66fe972dfc4267458783", "us-bis-export-7f2bd212278962a3422ea337f4a3c48d89b32dd5", "us-bis-export-451dbff38586313accead9604ed19a829c697a0c", "us-bis-export-db7e4415c40f144b86ae7e80663f1ecb3881c3f0", "us-bis-export-6fc4f02e29c3ce6946bba5ab46d85e6ddbd52011", "us-bis-export-a436233d2c6c56d960ebeb75515ff472269af881", "us-bis-export-9544416209657983bc7001b37e9d51060e72c975", "us-bis-export-82946210a8ddd470012f452ceae625c911696185", "us-bis-export-c273c16bf1303dd4a5ff63495ce04d48fb684bc8", "us-bis-export-a26010f4fbdff031cfbdd506b0c5473ba960de7c", "us-bis-export-76c90086df375e179d659f91819baed6c68924e5", "us-bis-export-dcceee15992199faf14eaa560e50eed1ac08cbff", "us-bis-export-5cea7d6d73036aed3a9b84b3acbf2ab4da5a5894", "us-bis-export-40cd785444939a13431fc3c0043e48fb491a19eb", "us-bis-export-429c02d458e26a3481e118ac2c5c839067149dcb", "us-bis-export-1a9181e9257e6781077da912c08bb91341bf776c", "us-bis-export-f9fefa36e1f866d630ded91684f83a1b6706930d", "us-bis-export-304a2d6acccb011ca183d5f74eb09e2adb1b3f7a", "us-bis-export-2424eac5562e3affcd5d3bffd15bddf88174ccc6", "us-bis-export-cbb6d8ecb514e3ae89dcaa1ad8ca4e0f4a1d3a8c", "us-bis-export-35b933a4c0b21fb19e559d4e0dbf8eb803f7736e", "us-bis-export-d07aa04f8fddc24521918cbd3fa708a9aff6b70f", "us-bis-export-d6ace3d53c1f5a32f9b42d5191ab03efb00ca334", "us-bis-export-b567ef733ad59c447f4c37a0517c908ecaccb1a3", "us-bis-export-8f3a6f47d9a111ce430642008abc33d24ae2de0e", "us-bis-export-f406edccfacbefd295d97789ad1f04d4be950e5f", "us-bis-export-62390dd00f64cd145f6da993b7584bc6576bbc59", "us-bis-export-9fca9bb2f6eb7b7731bc17f0bfdbe5357d71b549", "us-bis-export-c898c0d259425509cbcff7d87255626129febe27"]</t>
+          <t>["us-bis-export-5cea7d6d73036aed3a9b84b3acbf2ab4da5a5894", "us-bis-export-9fca9bb2f6eb7b7731bc17f0bfdbe5357d71b549", "us-bis-export-2424eac5562e3affcd5d3bffd15bddf88174ccc6", "us-bis-export-c273c16bf1303dd4a5ff63495ce04d48fb684bc8", "us-bis-export-9544416209657983bc7001b37e9d51060e72c975", "us-bis-export-40cd785444939a13431fc3c0043e48fb491a19eb", "us-bis-export-f9fefa36e1f866d630ded91684f83a1b6706930d", "us-bis-export-d6ace3d53c1f5a32f9b42d5191ab03efb00ca334", "us-bis-export-dcceee15992199faf14eaa560e50eed1ac08cbff", "us-bis-export-d07aa04f8fddc24521918cbd3fa708a9aff6b70f", "us-bis-export-a5e2916444556c0a92de66fe972dfc4267458783", "us-bis-export-db7e4415c40f144b86ae7e80663f1ecb3881c3f0", "us-bis-export-82946210a8ddd470012f452ceae625c911696185", "us-bis-export-35b933a4c0b21fb19e559d4e0dbf8eb803f7736e", "us-bis-export-7f2bd212278962a3422ea337f4a3c48d89b32dd5", "us-bis-export-304a2d6acccb011ca183d5f74eb09e2adb1b3f7a", "us-bis-export-1a9181e9257e6781077da912c08bb91341bf776c", "us-bis-export-b567ef733ad59c447f4c37a0517c908ecaccb1a3", "us-bis-export-c898c0d259425509cbcff7d87255626129febe27", "us-bis-export-1f6b4cd4b222a77730cdc398d633455b1f54f068", "us-bis-export-a26010f4fbdff031cfbdd506b0c5473ba960de7c", "us-bis-export-451dbff38586313accead9604ed19a829c697a0c", "us-bis-export-62390dd00f64cd145f6da993b7584bc6576bbc59", "us-bis-export-f406edccfacbefd295d97789ad1f04d4be950e5f", "us-bis-export-a436233d2c6c56d960ebeb75515ff472269af881", "us-bis-export-8f3a6f47d9a111ce430642008abc33d24ae2de0e", "us-bis-export-1878696a0dfcc2b4df8fe4c1b4c18ea191d2379a", "us-bis-export-76c90086df375e179d659f91819baed6c68924e5", "us-bis-export-cbb6d8ecb514e3ae89dcaa1ad8ca4e0f4a1d3a8c", "us-bis-export-429c02d458e26a3481e118ac2c5c839067149dcb", "us-bis-export-6fc4f02e29c3ce6946bba5ab46d85e6ddbd52011"]</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -872,7 +872,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>["isin-RU000A102L46", "isin-RU000A102TX2", "isin-RU000A101K55", "isin-RU000A104UG1", "isin-RU000A103S55", "isin-RU000A103DD6", "isin-RU000A107H88", "isin-RU000A105Q14", "isin-RU000A105X15", "isin-RU000A107FF7", "isin-RU000A103UF5", "isin-RU000A106VR1", "isin-RU000A1086L6", "isin-RU000A1022A4", "isin-RU000A1075B0", "isin-RU000A106HD0", "isin-RU000A106482", "isin-RU000A101W10", "isin-RU000A102VH1", "isin-RU000A102440", "isin-RU000A106L83", "isin-RU000A1026K4", "isin-RU000A1089S5", "isin-RU000A102X34", "isin-RU000A103075", "isin-RU000A102U11", "isin-RU000A102R32", "isin-RU000A103B88", "isin-RU000A107D82", "isin-RU000A1085E3"]</t>
+          <t>["isin-RU000A103075", "isin-RU000A103B88", "isin-RU000A1089S5", "isin-RU000A103DD6", "isin-RU000A101K55", "isin-RU000A102TX2", "isin-RU000A103UF5", "isin-RU000A105X15", "isin-RU000A1075B0", "isin-RU000A107D82", "isin-RU000A102440", "isin-RU000A1085E3", "isin-RU000A107H88", "isin-RU000A1026K4", "isin-RU000A102X34", "isin-RU000A106VR1", "isin-RU000A107FF7", "isin-RU000A1022A4", "isin-RU000A101W10", "isin-RU000A103S55", "isin-RU000A106L83", "isin-RU000A104UG1", "isin-RU000A1086L6", "isin-RU000A102R32", "isin-RU000A102U11", "isin-RU000A106482", "isin-RU000A106HD0", "isin-RU000A102L46", "isin-RU000A105Q14", "isin-RU000A102VH1"]</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -898,7 +898,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>["us-bis-export-fec8679ca8682155494c6534a4ee5b21ff3b7f9d", "us-bis-export-c3784bbfd503e94dc14dec4604a7db7fea3a286b", "us-bis-export-65ba375c8e6f9e21c9f8362aeb4153162ecf0fa3", "us-bis-export-ca88d5cb40a7fa4b0250bbc0b73836a3adf91e53", "us-bis-export-fb77edb924adb6876a9eb963e1fee728d0f26d29", "us-bis-export-ee6a6e5af365fdab9dfdf4382496f828293787b8", "us-bis-export-56cd1b244736bd025ae02ba2bb3c42cf4f733360", "us-bis-export-cadaadb3ac5e8ef7a86f871335e4c2fdf76cd4c4", "us-bis-export-624b97a8603a7ef546c92a35c4d3e5af1d3cc876", "us-bis-export-f4ff7f96cc5933c7c792a69eb76f13e6d555276f", "us-bis-export-06828ca4f4352159d0852bc986b8c3f289ef3f51", "us-bis-export-8c51d1e6c48e218a993a6720102d00df4e2408ec", "us-bis-export-4b8628aefdd6624df65a4477ea628b9f3a2af0b4", "us-bis-export-7b39486b819d36e8a9aa6fd1d68825ebfcb30458", "us-bis-export-a81c6ecf08dc8f41ea6ba548054e8b87e9b97b43", "us-bis-export-50cc107b01da267da5a31d838e32cc3d4c65c52e", "us-bis-export-6201250cfe17b557bda528f743f53f9049a438a8", "us-bis-export-a62f88117e7a420904e2b0a06c4e7b256c594e52", "us-bis-export-410c573386c9014d71542333965e0712707af209", "us-bis-export-01ae5f53cb8631efd22c90634e6b3f0daf2b31f4", "us-bis-export-6730408c0d53c0074ee6156b980c3c96a4de249e", "us-bis-export-6b68e59a1ea2c1e4fc58700e0e539bf48fd569e7", "us-bis-export-9a6860735e4fe52c2be61d3c2a950cb1ab0f3e2d", "us-bis-export-383cff5848ac7f218f43781e941b0138efe4f0a6", "us-bis-export-f393a6b2d87c456e8d74cc3269c4e3ee7e7e6ee8", "us-bis-export-7d393aff5c5b87ee72a9545b088f8d98844d68c2", "us-bis-export-56c858a23bf62b610bbbcfbd8a7b78895c04579b", "us-bis-export-2b378b31be5be3d7cfe08ef29e5b894c837ccb86", "us-bis-export-57dea62331f8c2e7af9b5625b136ff9862259408", "us-bis-export-7463531a400c15127b969e23180cf9a82edb5cb6"]</t>
+          <t>["us-bis-export-50cc107b01da267da5a31d838e32cc3d4c65c52e", "us-bis-export-01ae5f53cb8631efd22c90634e6b3f0daf2b31f4", "us-bis-export-383cff5848ac7f218f43781e941b0138efe4f0a6", "us-bis-export-2b378b31be5be3d7cfe08ef29e5b894c837ccb86", "us-bis-export-4b8628aefdd6624df65a4477ea628b9f3a2af0b4", "us-bis-export-56cd1b244736bd025ae02ba2bb3c42cf4f733360", "us-bis-export-f393a6b2d87c456e8d74cc3269c4e3ee7e7e6ee8", "us-bis-export-7463531a400c15127b969e23180cf9a82edb5cb6", "us-bis-export-fec8679ca8682155494c6534a4ee5b21ff3b7f9d", "us-bis-export-65ba375c8e6f9e21c9f8362aeb4153162ecf0fa3", "us-bis-export-6b68e59a1ea2c1e4fc58700e0e539bf48fd569e7", "us-bis-export-8c51d1e6c48e218a993a6720102d00df4e2408ec", "us-bis-export-f4ff7f96cc5933c7c792a69eb76f13e6d555276f", "us-bis-export-9a6860735e4fe52c2be61d3c2a950cb1ab0f3e2d", "us-bis-export-6730408c0d53c0074ee6156b980c3c96a4de249e", "us-bis-export-624b97a8603a7ef546c92a35c4d3e5af1d3cc876", "us-bis-export-a62f88117e7a420904e2b0a06c4e7b256c594e52", "us-bis-export-6201250cfe17b557bda528f743f53f9049a438a8", "us-bis-export-fb77edb924adb6876a9eb963e1fee728d0f26d29", "us-bis-export-7b39486b819d36e8a9aa6fd1d68825ebfcb30458", "us-bis-export-56c858a23bf62b610bbbcfbd8a7b78895c04579b", "us-bis-export-cadaadb3ac5e8ef7a86f871335e4c2fdf76cd4c4", "us-bis-export-410c573386c9014d71542333965e0712707af209", "us-bis-export-a81c6ecf08dc8f41ea6ba548054e8b87e9b97b43", "us-bis-export-c3784bbfd503e94dc14dec4604a7db7fea3a286b", "us-bis-export-57dea62331f8c2e7af9b5625b136ff9862259408", "us-bis-export-7d393aff5c5b87ee72a9545b088f8d98844d68c2", "us-bis-export-06828ca4f4352159d0852bc986b8c3f289ef3f51", "us-bis-export-ca88d5cb40a7fa4b0250bbc0b73836a3adf91e53", "us-bis-export-ee6a6e5af365fdab9dfdf4382496f828293787b8"]</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -924,7 +924,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>["us-bis-export-264ec488b29d10deb039c247b8496208b7397ace", "us-bis-export-647c6830d2826b8cd845c42a5eae9946429bdc86", "us-bis-export-5c00d8e1a29d0ae4c3146ad227436b1eb4f6450a", "us-bis-export-29286f39362e16186ff66f43d824d7c149d0cf5e", "us-bis-export-e0218cee700092b2f6e9e01f38f88166dec80343", "us-bis-export-5c477c9119a9029785a81caaffd8b312366bb263", "us-bis-export-706620519ae8fb4a4f810db388260dd30a726c8e", "us-bis-export-82548c7060d832ddd7882f64487d9a448f17842d", "us-bis-export-4f57f38b7f9f60b8ef3808c3860f840fef4debdc", "us-bis-export-39df58af4c9b98953a93b20e4717f44a671de9be", "us-bis-export-9e62fb0688a129e7e96b9dff2d17b58b212f0f01", "us-bis-export-4e109e82fe18d47620c00dc09394a4ef4ed9da71", "us-bis-export-818e037bb2ded176db067dc33676e2a3f4d8f743", "us-bis-export-11c361b6153227df3d2e88a538cb8e1c38781e10", "us-bis-export-a83c03e85a008168cf2e0f6dd76eb708a5ae0197", "us-bis-export-c3323518637a543be9fac0aab0cdc6ae8efd7814", "us-bis-export-39a6126126def4ea71a8893ca31d8ed2ddea624e", "us-bis-export-7b8d4306cbdf967e6b1418ff9b8d7cbbf2487f3f", "us-bis-export-21af2fdba43d96b925a0f037798cfbf6210e125c", "us-bis-export-feaf8da9b888e9080c6e4b361159ee272edb8798", "us-bis-export-b4c8aa4ca313e77b4d9ed20daa9c74bc9bd0cc53", "us-bis-export-36009800af7c39398369bfb9bb81d15a0b3db475", "us-bis-export-4264a0e89e0393d46b2582026729a197345799b6", "us-bis-export-a64597da05d34f192cf95bcb90fb58e6cac1652f", "us-bis-export-b6a264525172d04cd3d2b4609777b90358477b43", "us-bis-export-f12a0e20903f165eca9af99697055b33105a9736", "us-bis-export-26d6fe1a73312236b6ad7548adea92b51141da62", "us-bis-export-c1e49f54dbce7c0453458badad6ac55f0021cffd"]</t>
+          <t>["us-bis-export-5c00d8e1a29d0ae4c3146ad227436b1eb4f6450a", "us-bis-export-e0218cee700092b2f6e9e01f38f88166dec80343", "us-bis-export-36009800af7c39398369bfb9bb81d15a0b3db475", "us-bis-export-4f57f38b7f9f60b8ef3808c3860f840fef4debdc", "us-bis-export-39df58af4c9b98953a93b20e4717f44a671de9be", "us-bis-export-647c6830d2826b8cd845c42a5eae9946429bdc86", "us-bis-export-b6a264525172d04cd3d2b4609777b90358477b43", "us-bis-export-5c477c9119a9029785a81caaffd8b312366bb263", "us-bis-export-21af2fdba43d96b925a0f037798cfbf6210e125c", "us-bis-export-f12a0e20903f165eca9af99697055b33105a9736", "us-bis-export-c3323518637a543be9fac0aab0cdc6ae8efd7814", "us-bis-export-29286f39362e16186ff66f43d824d7c149d0cf5e", "us-bis-export-264ec488b29d10deb039c247b8496208b7397ace", "us-bis-export-82548c7060d832ddd7882f64487d9a448f17842d", "us-bis-export-11c361b6153227df3d2e88a538cb8e1c38781e10", "us-bis-export-feaf8da9b888e9080c6e4b361159ee272edb8798", "us-bis-export-4e109e82fe18d47620c00dc09394a4ef4ed9da71", "us-bis-export-c1e49f54dbce7c0453458badad6ac55f0021cffd", "us-bis-export-a64597da05d34f192cf95bcb90fb58e6cac1652f", "us-bis-export-39a6126126def4ea71a8893ca31d8ed2ddea624e", "us-bis-export-9e62fb0688a129e7e96b9dff2d17b58b212f0f01", "us-bis-export-4264a0e89e0393d46b2582026729a197345799b6", "us-bis-export-7b8d4306cbdf967e6b1418ff9b8d7cbbf2487f3f", "us-bis-export-818e037bb2ded176db067dc33676e2a3f4d8f743", "us-bis-export-26d6fe1a73312236b6ad7548adea92b51141da62", "us-bis-export-a83c03e85a008168cf2e0f6dd76eb708a5ae0197", "us-bis-export-b4c8aa4ca313e77b4d9ed20daa9c74bc9bd0cc53", "us-bis-export-706620519ae8fb4a4f810db388260dd30a726c8e"]</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -950,7 +950,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>["us-occ-18479-first-national-bank", "us-occ-20214-first-national-bank", "us-occ-13830-first-national-bank", "us-occ-8205-first-national-bank", "NK-PQKV6m5qiHTwLDWU7iXqBn", "us-occ-17129-first-national-bank", "us-occ-18125-first-national-bank", "us-occ-12423-first-national-bank", "NK-RPrxx7QDMC48WoRtfsVSYZ", "us-occ-14163-first-national-bank", "us-occ-13170-first-national-bank", "us-occ-18787-first-national-bank", "us-occ-14146-first-national-bank", "us-occ-7647-first-national-bank", "us-occ-14012-first-national-bank", "NK-aHpDcBPsCBsGiDs3VB9FMV", "us-occ-11968-first-national-bank", "us-occ-7853-first-national-bank", "us-occ-14252-first-national-bank", "us-occ-10230-first-national-bank", "us-occ-13742-first-national-bank", "NK-hNd7gSkdsgEtc2Cu2ehWpY", "us-occ-21610-first-national-bank", "us-occ-17324-first-national-bank", "us-occ-17710-first-national-bank", "us-occ-3496-first-national-bank", "NK-VEUcR2WqX6PU6EAJe9248K"]</t>
+          <t>["us-occ-18125-first-national-bank", "NK-aHpDcBPsCBsGiDs3VB9FMV", "us-occ-7853-first-national-bank", "NK-hNd7gSkdsgEtc2Cu2ehWpY", "us-occ-12423-first-national-bank", "us-occ-3496-first-national-bank", "us-occ-14146-first-national-bank", "us-occ-7647-first-national-bank", "us-occ-8205-first-national-bank", "us-occ-13170-first-national-bank", "us-occ-14252-first-national-bank", "NK-RPrxx7QDMC48WoRtfsVSYZ", "us-occ-11968-first-national-bank", "us-occ-17324-first-national-bank", "us-occ-18479-first-national-bank", "us-occ-21610-first-national-bank", "NK-PQKV6m5qiHTwLDWU7iXqBn", "us-occ-10230-first-national-bank", "us-occ-14012-first-national-bank", "us-occ-17129-first-national-bank", "us-occ-17710-first-national-bank", "us-occ-20214-first-national-bank", "NK-VEUcR2WqX6PU6EAJe9248K", "us-occ-14163-first-national-bank", "us-occ-18787-first-national-bank", "us-occ-13830-first-national-bank", "us-occ-13742-first-national-bank"]</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -976,7 +976,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>["us-bis-export-dc14fce64c4e0344ef0aaf83892b632b61068731", "us-bis-export-a61e141b1d62ffa7e7a023963c919bc16973ad6a", "us-bis-export-06b4ca1f7407964e2eba031e7e7c71ce709bf5cb", "us-bis-export-fedf7749dac3e962046a9dd7f2a16eb1664d1564", "us-bis-export-bf74de0594ae191f4f89580009eecd148fcf50c0", "us-bis-export-8776a0f9f9a1b5d1b562f062afa4a3d92b28a4ac", "us-bis-export-218a8dc6b04ba337c56129a9b165ebfe49a27a24", "us-bis-export-3c6e2c91f157b087fa544e2497b6a8a90f907b41", "us-bis-export-5edd5ab23cf265aa0a67b045caa2f8eadf834601", "us-bis-export-17ad59fc4ad80c3eca72d9d1960843b8a8705b61", "us-bis-export-a72b992940743df5f0a6f4ccb0f1e08291cf1778", "us-bis-export-e25dae8aa140bb74e933673805dd812947f804f9", "us-bis-export-0a6a060300638f2e79b43e087850dc51f22817b5", "us-bis-export-45f6f4d88223f01f73d042e6d82e278da68f3c2a", "us-bis-export-4e4521de256e257e56ef540cfc9615fbca58ffd5", "us-bis-export-3d1c12f3588b6b7bc5465a3ab8fa5b1881450ccf", "us-bis-export-afb52eaf128f3585a1175a56f1a28ec428feda70", "us-bis-export-a295516ab84e22c1ca78728dbf583db0ada3a5ee", "us-bis-export-2d2c0e1138134465184f8329dd9a9e2bd488eaea", "us-bis-export-281fab4da84b7335092ecd16a3ce755c7f9eaae7", "us-bis-export-bb54c8f154f6d8ce4de98322c2dfbddf266fb061", "us-bis-export-3b4d4492559520a3a05364d87c5eb1ece6a3d45a", "us-bis-export-9e4ddd0e1750640de0b220a6e2d0dadf485ce945", "us-bis-export-173fea845bf18b35427a8c7824154f304ae92699", "us-bis-export-85dd67671800490ba3681fb8ad28d2e8b105b77f", "us-bis-export-1404eb90b660ca2d82253d519bfae2c4b99c6d43", "us-bis-export-31b7a14650406324db7fb583916ff654aa71ad0d"]</t>
+          <t>["us-bis-export-4e4521de256e257e56ef540cfc9615fbca58ffd5", "us-bis-export-8776a0f9f9a1b5d1b562f062afa4a3d92b28a4ac", "us-bis-export-31b7a14650406324db7fb583916ff654aa71ad0d", "us-bis-export-a61e141b1d62ffa7e7a023963c919bc16973ad6a", "us-bis-export-9e4ddd0e1750640de0b220a6e2d0dadf485ce945", "us-bis-export-3c6e2c91f157b087fa544e2497b6a8a90f907b41", "us-bis-export-dc14fce64c4e0344ef0aaf83892b632b61068731", "us-bis-export-281fab4da84b7335092ecd16a3ce755c7f9eaae7", "us-bis-export-45f6f4d88223f01f73d042e6d82e278da68f3c2a", "us-bis-export-218a8dc6b04ba337c56129a9b165ebfe49a27a24", "us-bis-export-a72b992940743df5f0a6f4ccb0f1e08291cf1778", "us-bis-export-bf74de0594ae191f4f89580009eecd148fcf50c0", "us-bis-export-1404eb90b660ca2d82253d519bfae2c4b99c6d43", "us-bis-export-85dd67671800490ba3681fb8ad28d2e8b105b77f", "us-bis-export-fedf7749dac3e962046a9dd7f2a16eb1664d1564", "us-bis-export-bb54c8f154f6d8ce4de98322c2dfbddf266fb061", "us-bis-export-173fea845bf18b35427a8c7824154f304ae92699", "us-bis-export-2d2c0e1138134465184f8329dd9a9e2bd488eaea", "us-bis-export-06b4ca1f7407964e2eba031e7e7c71ce709bf5cb", "us-bis-export-5edd5ab23cf265aa0a67b045caa2f8eadf834601", "us-bis-export-e25dae8aa140bb74e933673805dd812947f804f9", "us-bis-export-3d1c12f3588b6b7bc5465a3ab8fa5b1881450ccf", "us-bis-export-17ad59fc4ad80c3eca72d9d1960843b8a8705b61", "us-bis-export-3b4d4492559520a3a05364d87c5eb1ece6a3d45a", "us-bis-export-a295516ab84e22c1ca78728dbf583db0ada3a5ee", "us-bis-export-0a6a060300638f2e79b43e087850dc51f22817b5", "us-bis-export-afb52eaf128f3585a1175a56f1a28ec428feda70"]</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>["isin-RU000A106JZ9", "isin-RU000A102VW0", "isin-RU000A107KV4", "isin-RU000A106K27", "isin-RU000A101XH9", "isin-RU000A1078H1", "isin-RU000A107AG6", "isin-RU000A105M75", "isin-RU000A106UW3", "isin-RU000A103UY6", "isin-RU000A105AW7", "isin-RU000A103FP5", "isin-RU000A103KJ8", "isin-RU000A106656", "isin-RU000A105492", "isin-RU000A105SX7", "isin-RU000A107456", "isin-RU000A106SE5", "isin-RU000A104ZV9", "isin-RU000A1030X9", "isin-RU000A105M91", "isin-RU000A104W58", "isin-RU000A107217", "isin-RU000A104JB5", "isin-RU000A105CM4", "isin-RU000A101YD6"]</t>
+          <t>["isin-RU000A106656", "isin-RU000A107456", "isin-RU000A1030X9", "isin-RU000A103KJ8", "isin-RU000A105M75", "isin-RU000A105CM4", "isin-RU000A102VW0", "isin-RU000A101YD6", "isin-RU000A106JZ9", "isin-RU000A106K27", "isin-RU000A104ZV9", "isin-RU000A104JB5", "isin-RU000A103UY6", "isin-RU000A107AG6", "isin-RU000A106SE5", "isin-RU000A106UW3", "isin-RU000A105SX7", "isin-RU000A107217", "isin-RU000A105492", "isin-RU000A105M91", "isin-RU000A104W58", "isin-RU000A103FP5", "isin-RU000A107KV4", "isin-RU000A1078H1", "isin-RU000A101XH9", "isin-RU000A105AW7"]</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>["isin-RU000A101QE0", "isin-RU000A103BQ2", "isin-RU000A10D4Y2", "isin-RU000A10BVH7", "isin-RU000A108EF8", "isin-RU000A106E90", "isin-RU000A10CKT3", "isin-RU000A10D517", "isin-RU000A108EG6", "isin-RU000A1028E3", "isin-RU000A1038Z7", "isin-RU000A1014N4", "isin-RU000A108EH4", "isin-RU000A1038V6", "isin-RU000A1074G2", "isin-RU000A108EE1", "isin-RU000A105FZ9", "isin-RU000A10BVC8", "isin-RU000A101F94", "isin-RU000A10D533", "isin-RU000A101FA1", "isin-RU000A105RV3", "isin-RU000A103901", "isin-RU000A103BR0", "isin-RU000A102BT8"]</t>
+          <t>["isin-RU000A105RV3", "isin-RU000A10BVC8", "isin-RU000A108EE1", "isin-RU000A10D517", "isin-RU000A108EG6", "isin-RU000A1028E3", "isin-RU000A10D533", "isin-RU000A1014N4", "isin-RU000A10D4Y2", "isin-RU000A101QE0", "isin-RU000A101FA1", "isin-RU000A10CKT3", "isin-RU000A1038Z7", "isin-RU000A106E90", "isin-RU000A102BT8", "isin-RU000A1074G2", "isin-RU000A101F94", "isin-RU000A103BQ2", "isin-RU000A105FZ9", "isin-RU000A103BR0", "isin-RU000A108EF8", "isin-RU000A103901", "isin-RU000A1038V6", "isin-RU000A10BVH7", "isin-RU000A108EH4"]</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>["isin-RU000A10A6W4", "isin-RU000A10DSU2", "isin-RU000A10EG28", "isin-RU000A107QM0", "isin-RU000A107U65", "isin-RU000A108AK6", "isin-RU000A10CZ43", "isin-RU000A10BV55", "isin-RU000A10B008", "isin-RU000A10B396", "isin-RU000A10C741", "isin-RU000A10DEE6", "isin-RU000A10CCJ1", "isin-RU000A10ASQ6", "isin-RU000A10C5J1", "isin-RU000A10DPT0", "isin-RU000A10B4U2", "isin-RU000A10B3A6", "isin-RU000A106QS9", "isin-RU000A10AXP8", "isin-RU000A10CZ35", "isin-RU000A107ST1", "isin-RU000A1082Y8", "isin-RU000A10BS76", "isin-RU000A10C5L7"]</t>
+          <t>["isin-RU000A10DSU2", "isin-RU000A10EG28", "isin-RU000A10B3A6", "isin-RU000A107ST1", "isin-RU000A10AXP8", "isin-RU000A107QM0", "isin-RU000A1082Y8", "isin-RU000A10B4U2", "isin-RU000A107U65", "isin-RU000A108AK6", "isin-RU000A10DEE6", "isin-RU000A106QS9", "isin-RU000A10BV55", "isin-RU000A10A6W4", "isin-RU000A10BS76", "isin-RU000A10C5J1", "isin-RU000A10DPT0", "isin-RU000A10ASQ6", "isin-RU000A10C741", "isin-RU000A10CCJ1", "isin-RU000A10CZ35", "isin-RU000A10B396", "isin-RU000A10C5L7", "isin-RU000A10B008", "isin-RU000A10CZ43"]</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>["isin-RU000A10B933", "isin-RU000A107WD7", "isin-RU000A10BJ02", "isin-RU000A10EKZ6", "isin-RU000A10BWC6", "isin-RU000A10AXW4", "isin-RU000A10CRP6", "isin-RU000A10B0S4", "isin-RU000A107QL2", "isin-RU000A109UD7", "isin-RU000A10ARS4", "isin-RU000A10C8M9", "isin-RU000A1080Y2", "isin-RU000A10DB16", "isin-RU000A109LC8", "isin-RU000A10BXV4", "isin-RU000A10E7K3", "isin-RU000A107SH6", "isin-RU000A10AZF4", "isin-RU000A10AUX8", "isin-RU000A10B3T6", "isin-RU000A109VK0", "isin-RU000A10BTQ2", "isin-RU000A107S85", "isin-RU000A109HX2"]</t>
+          <t>["isin-RU000A109VK0", "isin-RU000A107QL2", "isin-RU000A10AXW4", "isin-RU000A10AZF4", "isin-RU000A10E7K3", "isin-RU000A109HX2", "isin-RU000A107S85", "isin-RU000A1080Y2", "isin-RU000A10C8M9", "isin-RU000A10ARS4", "isin-RU000A109UD7", "isin-RU000A10AUX8", "isin-RU000A10B0S4", "isin-RU000A10BWC6", "isin-RU000A10EKZ6", "isin-RU000A107WD7", "isin-RU000A10B3T6", "isin-RU000A109LC8", "isin-RU000A10CRP6", "isin-RU000A10DB16", "isin-RU000A10B933", "isin-RU000A10BTQ2", "isin-RU000A10BXV4", "isin-RU000A10BJ02", "isin-RU000A107SH6"]</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>["no-nbim-46ac91a077b6c024128c2c2b2f0f03f37db76c42", "no-nbim-04113b29457e7dd9a46c0166be5f17ea12e448ea", "no-nbim-20325ad3083d0ff8ad422af46d970bc66fd2df4a", "no-nbim-4a220402953f34cd56e50670864f1de02710d28e", "no-nbim-37d6a36229c9644daa288e26ac0923c46003e01d", "no-nbim-4252715357037c18d58d2ec275d620657ec6cc8e", "no-nbim-7b5a5352f3a4d0bd7ebc83af08d513b439e3fbe9", "no-nbim-14d5b73c7448e6d23a8af79484167db48f96cabb", "no-nbim-d406f451b7171f33a4496dc638b1495fcf54ba65", "no-nbim-f2bb9fef70fcf9962dce52d7cda87123a39fedcb", "no-nbim-a4d6faf199e47ddaa804fe8a6d9f0a8c8c71e58a", "no-nbim-43b691c38cd2ba339a26370b3960886320701a8f", "no-nbim-54168605e905203ee16aa68cba04b6feba01f66e", "no-nbim-1977f3a41fc08cbc33794ef56f2e91e8943f6f84", "no-nbim-1e79f156fa7cbe04326ed3df5d7f137bc9b57964", "no-nbim-0c136825e3af083f0041685169e4a57c3e3466a7", "no-nbim-6842761b1f94e36a84558e70e02d51bbc026b7c8", "no-nbim-b85fe1c47acee66b1e7dd5f1a9df6dc26bea3b85", "no-nbim-0ee27d2d2189180162392c67cb1ecc5b711bc804", "no-nbim-86df20911ff88d155973ba77ca148a0bf531cc22", "no-nbim-2f7771e2b01547c1ed051a0f29af54fa0c96233e", "no-nbim-54a19ec5707a9151128df444880be1ee95ba4aa7", "no-nbim-dd4670872c7a1bc4a436d29402707fcd63b990ab", "no-nbim-7825269fe6f067176238eb2339e7206ffcc151e8", "no-nbim-80cf25833ca330c5a9011cd13aaac889ce7e3769"]</t>
+          <t>["no-nbim-0ee27d2d2189180162392c67cb1ecc5b711bc804", "no-nbim-f2bb9fef70fcf9962dce52d7cda87123a39fedcb", "no-nbim-d406f451b7171f33a4496dc638b1495fcf54ba65", "no-nbim-7b5a5352f3a4d0bd7ebc83af08d513b439e3fbe9", "no-nbim-04113b29457e7dd9a46c0166be5f17ea12e448ea", "no-nbim-46ac91a077b6c024128c2c2b2f0f03f37db76c42", "no-nbim-b85fe1c47acee66b1e7dd5f1a9df6dc26bea3b85", "no-nbim-80cf25833ca330c5a9011cd13aaac889ce7e3769", "no-nbim-37d6a36229c9644daa288e26ac0923c46003e01d", "no-nbim-dd4670872c7a1bc4a436d29402707fcd63b990ab", "no-nbim-54a19ec5707a9151128df444880be1ee95ba4aa7", "no-nbim-86df20911ff88d155973ba77ca148a0bf531cc22", "no-nbim-0c136825e3af083f0041685169e4a57c3e3466a7", "no-nbim-2f7771e2b01547c1ed051a0f29af54fa0c96233e", "no-nbim-20325ad3083d0ff8ad422af46d970bc66fd2df4a", "no-nbim-14d5b73c7448e6d23a8af79484167db48f96cabb", "no-nbim-4252715357037c18d58d2ec275d620657ec6cc8e", "no-nbim-4a220402953f34cd56e50670864f1de02710d28e", "no-nbim-1e79f156fa7cbe04326ed3df5d7f137bc9b57964", "no-nbim-43b691c38cd2ba339a26370b3960886320701a8f", "no-nbim-6842761b1f94e36a84558e70e02d51bbc026b7c8", "no-nbim-54168605e905203ee16aa68cba04b6feba01f66e", "no-nbim-a4d6faf199e47ddaa804fe8a6d9f0a8c8c71e58a", "no-nbim-1977f3a41fc08cbc33794ef56f2e91e8943f6f84", "no-nbim-7825269fe6f067176238eb2339e7206ffcc151e8"]</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>["isin-RU000A10EMT5", "isin-RU000A107SG8", "isin-RU000A10DCE0", "isin-RU000A109SJ8", "isin-RU000A10C6M3", "isin-RU000A10CH03", "isin-RU000A10BHY1", "isin-RU000A10BTT6", "isin-RU000A10E291", "isin-RU000A10AHB1", "isin-RU000A10DYB0", "isin-RU000A10ED62", "isin-RU000A10AC67", "isin-RU000A10A398", "isin-RU000A107R29", "isin-RU000A1099E4", "isin-RU000A10E7U2", "isin-RU000A10DE54", "isin-RU000A10DY84", "isin-RU000A1099W6", "isin-RU000A10B2P6", "isin-RU000A10EG44", "isin-RU000A10BQX4", "isin-RU000A10D4W6"]</t>
+          <t>["isin-RU000A10AC67", "isin-RU000A10BQX4", "isin-RU000A10D4W6", "isin-RU000A10C6M3", "isin-RU000A10E291", "isin-RU000A109SJ8", "isin-RU000A10DY84", "isin-RU000A10E7U2", "isin-RU000A107SG8", "isin-RU000A10AHB1", "isin-RU000A10DYB0", "isin-RU000A10B2P6", "isin-RU000A10DE54", "isin-RU000A10EMT5", "isin-RU000A10BHY1", "isin-RU000A107R29", "isin-RU000A10BTT6", "isin-RU000A10EG44", "isin-RU000A10ED62", "isin-RU000A10A398", "isin-RU000A10CH03", "isin-RU000A1099W6", "isin-RU000A10DCE0", "isin-RU000A1099E4"]</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>["sg-gov-a93e63023e86ca5386b8bb23dd755c74bbc95e50", "sg-gov-9a96fd0bf768a09822c966b7b44eb5e76a6934b9", "sg-gov-fd12b676f4351cdfc9dc60d1e79e93415a4eb3dc", "sg-gov-c829f977424d64b7986e37d0be7a7b6e3ad0523e", "sg-gov-64fa8dfbe7b96401b8b33a848c18220bb9b9e9e6", "sg-gov-4d6ca2a0fc046c0616ff2b69bd0c0c9c4485b16e", "sg-gov-db6ee8c9d9074ae4e4e5e785f197b92c2ebc147b", "sg-gov-9814022a95cd6bc0beea8501d4e10f03738a84dc", "sg-gov-cf2dd9d128ecec72bf3b44af1dce9953666281d1", "sg-gov-1927ac2500e15defba3f881a7bb6a848c4d567dd", "sg-gov-794729f23280383e04b16a261c769042e33ed6a9", "sg-gov-614c74afa47eced172ed3f668fff503e229ce552", "sg-gov-ae9e3a5efb2b35f3205437449cd0adfd719c8bf9", "sg-gov-d1a6df395955e8a6877de5a6cda9bc290e46101d", "sg-gov-5e39ca8dd413db5428515dc7a00494bdd4da858e", "sg-gov-94fc488595eb577cd6ba2705b92c3482b4e02425", "sg-gov-2fc6f733cd9085bef8aee4dde734b49e392b4c85", "sg-gov-013e1d8d8032a9c7bc6036919935f2b093af042b", "sg-gov-d1bca9c114e1a89a6512eb125e6c59a40672f237", "sg-gov-3301993066bbd63cd5afc2e1d176a34c5d36dfcd", "sg-gov-62f44c94332d3be8bc8cff76681436955dec35f4", "sg-gov-2580ce11f24ca1d0d4874fc5969477fb433fec20", "sg-gov-828fcb00f515ba3853dd3753b352841cafead58d", "sg-gov-0019b5723ae2b3bab694a56a064525cb3e070196"]</t>
+          <t>["sg-gov-9814022a95cd6bc0beea8501d4e10f03738a84dc", "sg-gov-db6ee8c9d9074ae4e4e5e785f197b92c2ebc147b", "sg-gov-794729f23280383e04b16a261c769042e33ed6a9", "sg-gov-828fcb00f515ba3853dd3753b352841cafead58d", "sg-gov-62f44c94332d3be8bc8cff76681436955dec35f4", "sg-gov-013e1d8d8032a9c7bc6036919935f2b093af042b", "sg-gov-ae9e3a5efb2b35f3205437449cd0adfd719c8bf9", "sg-gov-5e39ca8dd413db5428515dc7a00494bdd4da858e", "sg-gov-2fc6f733cd9085bef8aee4dde734b49e392b4c85", "sg-gov-fd12b676f4351cdfc9dc60d1e79e93415a4eb3dc", "sg-gov-4d6ca2a0fc046c0616ff2b69bd0c0c9c4485b16e", "sg-gov-d1a6df395955e8a6877de5a6cda9bc290e46101d", "sg-gov-64fa8dfbe7b96401b8b33a848c18220bb9b9e9e6", "sg-gov-cf2dd9d128ecec72bf3b44af1dce9953666281d1", "sg-gov-3301993066bbd63cd5afc2e1d176a34c5d36dfcd", "sg-gov-a93e63023e86ca5386b8bb23dd755c74bbc95e50", "sg-gov-614c74afa47eced172ed3f668fff503e229ce552", "sg-gov-c829f977424d64b7986e37d0be7a7b6e3ad0523e", "sg-gov-2580ce11f24ca1d0d4874fc5969477fb433fec20", "sg-gov-d1bca9c114e1a89a6512eb125e6c59a40672f237", "sg-gov-0019b5723ae2b3bab694a56a064525cb3e070196", "sg-gov-1927ac2500e15defba3f881a7bb6a848c4d567dd", "sg-gov-94fc488595eb577cd6ba2705b92c3482b4e02425", "sg-gov-9a96fd0bf768a09822c966b7b44eb5e76a6934b9"]</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>["isin-RU000A103QK3", "isin-RU000A106P63", "isin-RU000A102200", "isin-RU000A1060X6", "isin-RU000A102KU7", "isin-RU000A106UM4", "isin-RU000A107GV2", "isin-RU000A102B48", "isin-RU000A102T97", "isin-RU000A102J57", "isin-RU000A106U90", "isin-RU000A105Q89", "isin-RU000A105WC3", "isin-RU000A107001", "isin-RU000A105XF4", "isin-RU000A106HF5", "isin-RU000A1074Q1", "isin-RU000A1022G1", "isin-RU000A1060Q0", "isin-RU000A1043Z7", "isin-RU000A103CD8", "isin-RU000A102AK9"]</t>
+          <t>["isin-RU000A105Q89", "isin-RU000A107001", "isin-RU000A102B48", "isin-RU000A103CD8", "isin-RU000A1043Z7", "isin-RU000A102KU7", "isin-RU000A102200", "isin-RU000A1074Q1", "isin-RU000A107GV2", "isin-RU000A1060Q0", "isin-RU000A1022G1", "isin-RU000A103QK3", "isin-RU000A106U90", "isin-RU000A106P63", "isin-RU000A102J57", "isin-RU000A105XF4", "isin-RU000A102AK9", "isin-RU000A1060X6", "isin-RU000A102T97", "isin-RU000A106UM4", "isin-RU000A106HF5", "isin-RU000A105WC3"]</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>["isin-RU000A10ADD6", "isin-RU000A108FS8", "isin-RU000A10A1N4", "isin-RU000A10DA58", "isin-RU000A1094W7", "isin-RU000A10B6K8", "isin-RU000A107W71", "isin-RU000A10B7S9", "isin-RU000A10BRY0", "isin-RU000A109QQ7", "isin-RU000A10E5Y8", "isin-RU000A10DD97", "isin-RU000A108E80", "isin-RU000A10E9M5", "isin-RU000A10B5M6", "isin-RU000A10CJ84", "isin-RU000A10EFW3", "isin-RU000A10B5A1", "isin-RU000A109R50", "isin-RU000A10DTU0", "isin-RU000A10DLY9", "isin-RU000A10CST6"]</t>
+          <t>["isin-RU000A10CJ84", "isin-RU000A10DA58", "isin-RU000A10DD97", "isin-RU000A10B6K8", "isin-RU000A109R50", "isin-RU000A10E5Y8", "isin-RU000A10ADD6", "isin-RU000A108FS8", "isin-RU000A10E9M5", "isin-RU000A109QQ7", "isin-RU000A10BRY0", "isin-RU000A10B7S9", "isin-RU000A108E80", "isin-RU000A10B5A1", "isin-RU000A10B5M6", "isin-RU000A10EFW3", "isin-RU000A10DLY9", "isin-RU000A1094W7", "isin-RU000A10CST6", "isin-RU000A107W71", "isin-RU000A10A1N4", "isin-RU000A10DTU0"]</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>["us-bis-export-b194b89e3edad175738bbf00c0a5d0aa04c32c7e", "us-bis-export-95e00cf9524edf302d6a5d8ada933810c3ef58bd", "us-bis-export-aa6ac67a6e6a0368faf3a4af1ae3926a5a160f48", "us-bis-export-67e260a57a8b4765a8569cf0b4dff53040d04aa1", "us-bis-export-ca81a679e19a211e7cfc19a8741fcdc6ab3f2bd8", "us-bis-export-8ab589564d10f1a1bfc884342d729d801365f078", "us-bis-export-31b5980d59cad15f717ea5a0f834828197a31378", "us-bis-export-0bcd76f3bae9b241d3fcb3af2ff43fab510e891c", "us-bis-export-d9c3f96987659b69729b05579ce9cb6f01d311ef", "us-bis-export-0bd4567190959cfc6a293f3406a6535040771c63", "us-bis-export-dc7b2e7354e58f567d74c8b82986427353a7217a", "us-bis-export-e0f6ec8632de4d5956e691705e14e11f9e966621", "us-bis-export-e9284d5d6ae34f203de5ae376a0e8aaa8b6b6d01", "us-bis-export-20bb29356a300e96fe7450126f4ddf9bd8af9eb4", "us-bis-export-bba74fdbbd08546826f71684bf523e17390b704c", "us-bis-export-b6d9a86e73c8a14cc3f69098c077f0a477bd50ff", "us-bis-export-5c42d11d5978ac49d3245471a4391a7a7f887cec", "us-bis-export-a78c7b4be367a59af55ba73a79de0e3ea863be11", "us-bis-export-070a9418024dc4c861eaaaa578715d281c579d20", "us-bis-export-99ce99a9d90710c2dac70c609aaeaea3943465c3", "us-bis-export-7b75563abace54b3750b066822080b27054e006b", "us-bis-export-f1871aecb94cc579532c623408bbd19d88d76a81"]</t>
+          <t>["us-bis-export-67e260a57a8b4765a8569cf0b4dff53040d04aa1", "us-bis-export-d9c3f96987659b69729b05579ce9cb6f01d311ef", "us-bis-export-b6d9a86e73c8a14cc3f69098c077f0a477bd50ff", "us-bis-export-b194b89e3edad175738bbf00c0a5d0aa04c32c7e", "us-bis-export-bba74fdbbd08546826f71684bf523e17390b704c", "us-bis-export-ca81a679e19a211e7cfc19a8741fcdc6ab3f2bd8", "us-bis-export-dc7b2e7354e58f567d74c8b82986427353a7217a", "us-bis-export-f1871aecb94cc579532c623408bbd19d88d76a81", "us-bis-export-0bd4567190959cfc6a293f3406a6535040771c63", "us-bis-export-070a9418024dc4c861eaaaa578715d281c579d20", "us-bis-export-20bb29356a300e96fe7450126f4ddf9bd8af9eb4", "us-bis-export-5c42d11d5978ac49d3245471a4391a7a7f887cec", "us-bis-export-31b5980d59cad15f717ea5a0f834828197a31378", "us-bis-export-0bcd76f3bae9b241d3fcb3af2ff43fab510e891c", "us-bis-export-e9284d5d6ae34f203de5ae376a0e8aaa8b6b6d01", "us-bis-export-7b75563abace54b3750b066822080b27054e006b", "us-bis-export-a78c7b4be367a59af55ba73a79de0e3ea863be11", "us-bis-export-aa6ac67a6e6a0368faf3a4af1ae3926a5a160f48", "us-bis-export-8ab589564d10f1a1bfc884342d729d801365f078", "us-bis-export-95e00cf9524edf302d6a5d8ada933810c3ef58bd", "us-bis-export-e0f6ec8632de4d5956e691705e14e11f9e966621", "us-bis-export-99ce99a9d90710c2dac70c609aaeaea3943465c3"]</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>["us-bis-export-a66c36ad213a6d3de23572c73c046d1f815365c2", "us-bis-export-838f40aae3d8c2c6b820d53373786da022bbad31", "us-bis-export-5c319d600981b5db3266bc71c1bbfb5138847a59", "us-bis-export-8f1d8eb816688c0121d436c54c8052c4adc31134", "us-bis-export-bfc72336fb63d1f44bab067cf035e93ede5f9678", "us-bis-export-ca6e412b1391ca54f63947807d98479d1a671f76", "us-bis-export-e61e6d2c7005b45d4aa26a0bf6838cdc2e1e0d06", "us-bis-export-bdbfcd189c60bb175c4239da0b539a4089b02c9d", "us-bis-export-bc925a30a4c841245755ea1080e11db9f5778918", "us-bis-export-eb93fd0e4e8300d577ae1d93ede9a4648b5b2e4f", "us-bis-export-751a34d9931eda6d59b0b01ebad576a04fe69c21", "us-bis-export-0f4075cdfaef34bc63acdebb7f28a331d4ba55e7", "us-bis-export-69d87f6441baaee676e8805be4a9c33a108e80cb", "us-bis-export-71bbfa7d8e06753f33eb55750f90f0b83900e650", "us-bis-export-460a88d54d1e453481b038cb41a8733fdb2f2748", "us-bis-export-2835c8b6ce5e23de2b1089574f821c2e8c35d636", "us-bis-export-2f4847eb6d7000565f5634ab49dbcb2529d7e52a", "us-bis-export-20809edf4fb94a271cfe4a46bfb2fe8289f1ff24", "us-bis-export-c612f655270fc0f7a1943e189575bc7c13cb171e", "us-bis-export-fae583b4d3b4960813de4e9898954dccc65307c1", "us-bis-export-cd23502eefc825a42b55ff0a4706a3e732059477", "us-bis-export-5011cf717c40b95c8c47561cee6035c9bf703ea8"]</t>
+          <t>["us-bis-export-fae583b4d3b4960813de4e9898954dccc65307c1", "us-bis-export-0f4075cdfaef34bc63acdebb7f28a331d4ba55e7", "us-bis-export-5011cf717c40b95c8c47561cee6035c9bf703ea8", "us-bis-export-69d87f6441baaee676e8805be4a9c33a108e80cb", "us-bis-export-2f4847eb6d7000565f5634ab49dbcb2529d7e52a", "us-bis-export-cd23502eefc825a42b55ff0a4706a3e732059477", "us-bis-export-bc925a30a4c841245755ea1080e11db9f5778918", "us-bis-export-e61e6d2c7005b45d4aa26a0bf6838cdc2e1e0d06", "us-bis-export-ca6e412b1391ca54f63947807d98479d1a671f76", "us-bis-export-c612f655270fc0f7a1943e189575bc7c13cb171e", "us-bis-export-71bbfa7d8e06753f33eb55750f90f0b83900e650", "us-bis-export-20809edf4fb94a271cfe4a46bfb2fe8289f1ff24", "us-bis-export-a66c36ad213a6d3de23572c73c046d1f815365c2", "us-bis-export-838f40aae3d8c2c6b820d53373786da022bbad31", "us-bis-export-bdbfcd189c60bb175c4239da0b539a4089b02c9d", "us-bis-export-eb93fd0e4e8300d577ae1d93ede9a4648b5b2e4f", "us-bis-export-460a88d54d1e453481b038cb41a8733fdb2f2748", "us-bis-export-bfc72336fb63d1f44bab067cf035e93ede5f9678", "us-bis-export-751a34d9931eda6d59b0b01ebad576a04fe69c21", "us-bis-export-5c319d600981b5db3266bc71c1bbfb5138847a59", "us-bis-export-2835c8b6ce5e23de2b1089574f821c2e8c35d636", "us-bis-export-8f1d8eb816688c0121d436c54c8052c4adc31134"]</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>["us-bis-export-495d5ef999a879ccf323201668b97b43bd2bebb2", "us-bis-export-6a2e184f7f129f3af838dde84fc883f7c8ed728e", "us-bis-export-bbdc1db8da8709558874164e7b0a5e77fbf670d2", "us-bis-export-5bc48fc45185208bfeafad3af72be80a0eb4cb7f", "us-bis-export-879c73573486390fa1393639d0277f7723f3abe4", "us-bis-export-d616b39ea7d079d489420297559be1ff62eded96", "us-bis-export-209182617447ec396edbd9f87bca3183a40ea2c6", "us-bis-export-d84f17b0e98705fcfcd6c07897d4add05a1f4404", "us-bis-export-c3645c67ae58b75aef7f8fd4797aa4cfa2d38c35", "us-bis-export-e359171f0ec9509c16f390dfab8be4664982edf2", "us-bis-export-e10f750a97f3e46190458feca8d78a9130ffca0c", "us-bis-export-a700af94468f7e84c736555b50e17764dbde29d3", "us-bis-export-45547edf9716ca47f9f50f7d4cfdc0b0c7b6c331", "us-bis-export-7cb9ddd92a5af29c594fb4805f8c6932988a2ed7", "us-bis-export-9acc1f3076edd878c7e9489d31a88b8fc99e004f", "us-bis-export-4bf84b55868526c30a4c95b516454f1b611be1a1", "us-bis-export-b95635194a5c1d4439d6efb227dfa1889142b79a", "us-bis-export-261df25e91433e816c44515004bb5f958d7fd06c", "us-bis-export-99df182ea8c36e108d01be191737ae533c11bbcf", "us-bis-export-d82dc72cb2cf2776e188f49912a409550a26d711", "us-bis-export-7e1dc1faeb06317f0b0e7003d7264536facdfce7", "us-bis-export-61b7348ec1e9088dc6b738dba3bbf5123faa65f7"]</t>
+          <t>["us-bis-export-7e1dc1faeb06317f0b0e7003d7264536facdfce7", "us-bis-export-d82dc72cb2cf2776e188f49912a409550a26d711", "us-bis-export-9acc1f3076edd878c7e9489d31a88b8fc99e004f", "us-bis-export-bbdc1db8da8709558874164e7b0a5e77fbf670d2", "us-bis-export-d616b39ea7d079d489420297559be1ff62eded96", "us-bis-export-209182617447ec396edbd9f87bca3183a40ea2c6", "us-bis-export-5bc48fc45185208bfeafad3af72be80a0eb4cb7f", "us-bis-export-a700af94468f7e84c736555b50e17764dbde29d3", "us-bis-export-45547edf9716ca47f9f50f7d4cfdc0b0c7b6c331", "us-bis-export-c3645c67ae58b75aef7f8fd4797aa4cfa2d38c35", "us-bis-export-b95635194a5c1d4439d6efb227dfa1889142b79a", "us-bis-export-261df25e91433e816c44515004bb5f958d7fd06c", "us-bis-export-d84f17b0e98705fcfcd6c07897d4add05a1f4404", "us-bis-export-99df182ea8c36e108d01be191737ae533c11bbcf", "us-bis-export-879c73573486390fa1393639d0277f7723f3abe4", "us-bis-export-495d5ef999a879ccf323201668b97b43bd2bebb2", "us-bis-export-e359171f0ec9509c16f390dfab8be4664982edf2", "us-bis-export-6a2e184f7f129f3af838dde84fc883f7c8ed728e", "us-bis-export-e10f750a97f3e46190458feca8d78a9130ffca0c", "us-bis-export-61b7348ec1e9088dc6b738dba3bbf5123faa65f7", "us-bis-export-7cb9ddd92a5af29c594fb4805f8c6932988a2ed7", "us-bis-export-4bf84b55868526c30a4c95b516454f1b611be1a1"]</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>["isin-RU000A108GM9", "isin-RU000A107UB5", "isin-RU000A10E6D0", "isin-RU000A10C9Y2", "isin-RU000A107U40", "isin-RU000A10D4P0", "isin-RU000A10A4C1", "isin-RU000A1097C2", "isin-RU000A108WV7", "isin-RU000A10B3X8", "isin-RU000A1082K7", "isin-RU000A10BJ85", "isin-RU000A10C5K9", "isin-RU000A107W06", "isin-RU000A10A6U8", "isin-RU000A10BWL7", "isin-RU000A10AV31", "isin-RU000A10B4W8", "isin-RU000A10B750", "isin-RU000A10B2X0", "isin-RU000A10BFG2"]</t>
+          <t>["isin-RU000A10B750", "isin-RU000A107W06", "isin-RU000A10BFG2", "isin-RU000A10B2X0", "isin-RU000A10BJ85", "isin-RU000A108GM9", "isin-RU000A10C5K9", "isin-RU000A108WV7", "isin-RU000A10AV31", "isin-RU000A107UB5", "isin-RU000A1082K7", "isin-RU000A10A4C1", "isin-RU000A10C9Y2", "isin-RU000A107U40", "isin-RU000A10E6D0", "isin-RU000A10A6U8", "isin-RU000A10B4W8", "isin-RU000A10D4P0", "isin-RU000A10B3X8", "isin-RU000A1097C2", "isin-RU000A10BWL7"]</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>["us-bis-export-74c75668144750df248c0934eeeda17cc295fa64", "us-bis-export-a932b66db5e2cb883f8e9f62795682a3d2793c0e", "us-bis-export-4f15715bfa15bb1d1bbbef4f26261b414354858e", "us-bis-export-d75a538d6160f8834824bbc8d7ca626d60de657e", "us-bis-export-020d0ffa4f3afcce77f012d727b467d317e7e9db", "us-bis-export-5944af2a6b2433236a79fa36d0f03dac37c06035", "us-bis-export-83b2b506e661eab620190113dbdb874c38992aef", "us-bis-export-66cea3a7fe3da5a638361f251fbd1a5e92b7d560", "us-bis-export-43caa771a65771f1fbb3c487692074dd99eae30d", "us-bis-export-f3381c93f958c84e2ccb561654155a8cfeebde71", "us-bis-export-e73bb9f346a85cba47fe1377ca0c12e881572cdb", "us-bis-export-62895e8eac035752ce9c8b9f895aa0df96368b9a", "us-bis-export-1fe7b1caf8fef630e7d824dc2b04745e6dd6256d", "us-bis-export-35ca9b34585a509b4da8a62069c5961dc9bcc934", "us-bis-export-539e60427aabf99c9c6c268d51e373b63f2e8a33", "us-bis-export-49eee0e9a1d21bd7b32e94ea237ccae74717742e", "us-bis-export-2603358c5b2f6847657a8972e20a62b24fe638c4", "us-bis-export-3ac4d5f3a4cf9c2c5f75fecd80455e5cfcce7492", "us-bis-export-8aaf946ddb3c987d32f2735fc1a3a1c58e4e7097", "us-bis-export-8b43476bc109335dcf2be663a2e6996e22762136", "us-bis-export-2d2e65a0f060212aee1ef47e581a7ac389202b8f"]</t>
+          <t>["us-bis-export-43caa771a65771f1fbb3c487692074dd99eae30d", "us-bis-export-1fe7b1caf8fef630e7d824dc2b04745e6dd6256d", "us-bis-export-4f15715bfa15bb1d1bbbef4f26261b414354858e", "us-bis-export-49eee0e9a1d21bd7b32e94ea237ccae74717742e", "us-bis-export-539e60427aabf99c9c6c268d51e373b63f2e8a33", "us-bis-export-62895e8eac035752ce9c8b9f895aa0df96368b9a", "us-bis-export-35ca9b34585a509b4da8a62069c5961dc9bcc934", "us-bis-export-f3381c93f958c84e2ccb561654155a8cfeebde71", "us-bis-export-8b43476bc109335dcf2be663a2e6996e22762136", "us-bis-export-5944af2a6b2433236a79fa36d0f03dac37c06035", "us-bis-export-020d0ffa4f3afcce77f012d727b467d317e7e9db", "us-bis-export-74c75668144750df248c0934eeeda17cc295fa64", "us-bis-export-2d2e65a0f060212aee1ef47e581a7ac389202b8f", "us-bis-export-a932b66db5e2cb883f8e9f62795682a3d2793c0e", "us-bis-export-e73bb9f346a85cba47fe1377ca0c12e881572cdb", "us-bis-export-83b2b506e661eab620190113dbdb874c38992aef", "us-bis-export-8aaf946ddb3c987d32f2735fc1a3a1c58e4e7097", "us-bis-export-3ac4d5f3a4cf9c2c5f75fecd80455e5cfcce7492", "us-bis-export-2603358c5b2f6847657a8972e20a62b24fe638c4", "us-bis-export-d75a538d6160f8834824bbc8d7ca626d60de657e", "us-bis-export-66cea3a7fe3da5a638361f251fbd1a5e92b7d560"]</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>["Q133820138", "Q116056196", "Q136745505", "Q137794235", "Q110070915", "Q116056211", "Q137595068", "Q30755529", "Q116056154", "Q28603835", "Q30723983", "Q136979359", "Q20500051", "Q133539204", "Q116055982", "Q116056259", "Q116056140", "Q34526819", "Q31192847"]</t>
+          <t>["Q30723983", "Q110070915", "Q133820138", "Q133539204", "Q137794235", "Q31192847", "Q116056259", "Q136745505", "Q116056196", "Q20500051", "Q137595068", "Q116055982", "Q116056211", "Q136979359", "Q34526819", "Q116056154", "Q30755529", "Q116056140", "Q28603835"]</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>["isin-RU000A1025A7", "isin-RU000A101KT1", "isin-RU000A105B11", "isin-RU000A106Z61", "isin-RU000A101N52", "isin-RU000A1028D5", "isin-RU000A102A49", "isin-RU000A102BV4", "isin-RU000A105L19", "isin-RU000A10A7D2", "isin-RU000A1025B5", "isin-RU000A10AA93", "isin-RU000A1066D5", "isin-RU000A10D4Z9", "isin-RU000A101CK7", "isin-RU000A10D525", "isin-RU000A105G16", "isin-RU000A102A31", "isin-RU000A100QS2"]</t>
+          <t>["isin-RU000A105L19", "isin-RU000A105B11", "isin-RU000A1025B5", "isin-RU000A1025A7", "isin-RU000A101KT1", "isin-RU000A10AA93", "isin-RU000A102BV4", "isin-RU000A10A7D2", "isin-RU000A102A31", "isin-RU000A1028D5", "isin-RU000A101N52", "isin-RU000A1066D5", "isin-RU000A105G16", "isin-RU000A100QS2", "isin-RU000A10D525", "isin-RU000A102A49", "isin-RU000A106Z61", "isin-RU000A101CK7", "isin-RU000A10D4Z9"]</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -1418,7 +1418,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>["isin-RU000A107BJ8", "isin-RU000A10EEU0", "isin-RU000A10EEL9", "isin-RU000A10C5X2", "isin-RU000A10AZ03", "isin-RU000A108K41", "isin-RU000A10BH04", "isin-RU000A10BT91", "isin-RU000A109P60", "isin-RU000A10DED8", "isin-RU000A10B7Z4", "isin-RU000A10C2G4", "isin-RU000A109817", "isin-RU000A10BH38", "isin-RU000A10BFU3", "isin-RU000A107UD1", "isin-RU000A10BH46", "isin-RU000A106664", "isin-RU000A10DKT1"]</t>
+          <t>["isin-RU000A109817", "isin-RU000A107UD1", "isin-RU000A10BH46", "isin-RU000A10EEL9", "isin-RU000A10EEU0", "isin-RU000A10DED8", "isin-RU000A10BFU3", "isin-RU000A108K41", "isin-RU000A10C5X2", "isin-RU000A10B7Z4", "isin-RU000A10C2G4", "isin-RU000A107BJ8", "isin-RU000A10BH38", "isin-RU000A106664", "isin-RU000A109P60", "isin-RU000A10BT91", "isin-RU000A10AZ03", "isin-RU000A10DKT1", "isin-RU000A10BH04"]</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>["isin-RU000A10E5U6", "isin-RU000A10AG89", "isin-RU000A10D1C4", "isin-RU000A10CRR2", "isin-RU000A10C2H2", "isin-RU000A109P94", "isin-RU000A108QN6", "isin-RU000A1099N5", "isin-RU000A10A3E9", "isin-RU000A109X60", "isin-RU000A10AP13", "isin-RU000A10A6S2", "isin-RU000A108PJ6", "isin-RU000A10B5K0", "isin-RU000A1099M7", "isin-RU000A10C3C1", "isin-RU000A10B7K6", "isin-RU000A109F47", "isin-RU000A10E9T0"]</t>
+          <t>["isin-RU000A109P94", "isin-RU000A10B5K0", "isin-RU000A10E9T0", "isin-RU000A10C2H2", "isin-RU000A1099N5", "isin-RU000A1099M7", "isin-RU000A109X60", "isin-RU000A10AG89", "isin-RU000A10AP13", "isin-RU000A108PJ6", "isin-RU000A10B7K6", "isin-RU000A109F47", "isin-RU000A10C3C1", "isin-RU000A10E5U6", "isin-RU000A10D1C4", "isin-RU000A10A3E9", "isin-RU000A108QN6", "isin-RU000A10CRR2", "isin-RU000A10A6S2"]</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>["ru-90a64ab6f595aac0813340722527e78e7ad65e7f", "ru-dbb1d6b680212b664c67ca872923a29b00ccf843", "ru-22b5dfc2c6f6845d5b336a501923b39963729da1", "ru-d33061f978495baf77808882721cda4dd668fb8f", "ru-02f79694ce8503cd32cc193dd09de6b3bc4bf71c", "ru-0b445022b0ec05fd6b34ae90e6f015a61ac43b32", "ru-1971ba12dbfff139a0eeaf75417a584b6e85d7e1", "ru-805da21ef189ec834359be7790272ba7891448bb", "ru-842769086a86a54eadd47780edad8d989983cb2e", "ru-e4d52d0d6e881b96b34c805407afd340b90e5286", "ru-c196c159eede00171714dbd1e44ff7e8f121be86", "ru-a94a261e1c395fd3f0b17b86415b4bece3d1fda7", "ru-f841eecb6dcfede6347f7e198fac0191abd62d9b", "ru-a3e8334bc3185ee1f3cda439c723355b9267abf3", "ru-2255f7116450b3310dc43e58341e7c6cd9795472", "ru-9e9eaa6fa8fb5f871e8dcf20f84e4d5b1f5aaff4", "ru-b97bd09714e6b296aa6b71f11508ead3c927428f", "ru-67ca0d489769b18c0a473e21a1b64de3b19cd356", "ru-79738a69df052b67aa260d4c1980aaad822f1c3c"]</t>
+          <t>["ru-b97bd09714e6b296aa6b71f11508ead3c927428f", "ru-e4d52d0d6e881b96b34c805407afd340b90e5286", "ru-02f79694ce8503cd32cc193dd09de6b3bc4bf71c", "ru-a94a261e1c395fd3f0b17b86415b4bece3d1fda7", "ru-c196c159eede00171714dbd1e44ff7e8f121be86", "ru-842769086a86a54eadd47780edad8d989983cb2e", "ru-2255f7116450b3310dc43e58341e7c6cd9795472", "ru-22b5dfc2c6f6845d5b336a501923b39963729da1", "ru-79738a69df052b67aa260d4c1980aaad822f1c3c", "ru-a3e8334bc3185ee1f3cda439c723355b9267abf3", "ru-9e9eaa6fa8fb5f871e8dcf20f84e4d5b1f5aaff4", "ru-1971ba12dbfff139a0eeaf75417a584b6e85d7e1", "ru-0b445022b0ec05fd6b34ae90e6f015a61ac43b32", "ru-90a64ab6f595aac0813340722527e78e7ad65e7f", "ru-805da21ef189ec834359be7790272ba7891448bb", "ru-d33061f978495baf77808882721cda4dd668fb8f", "ru-f841eecb6dcfede6347f7e198fac0191abd62d9b", "ru-dbb1d6b680212b664c67ca872923a29b00ccf843", "ru-67ca0d489769b18c0a473e21a1b64de3b19cd356"]</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>["isin-RU000A102770", "isin-RU000A101R74", "isin-RU000A102FD3", "isin-RU000A101KR5", "isin-RU000A102BC4", "isin-RU000A102Q90", "isin-RU000A102SL9", "isin-RU000A102YY0", "isin-RU000A102374", "isin-RU000A1036C0", "isin-RU000A103MY3", "isin-RU000A101MQ3", "isin-RU000A103232", "isin-RU000A101ZK8", "isin-RU000A103D60", "isin-RU000A101UM5", "isin-RU000A103GZ2", "isin-RU000A102MW9"]</t>
+          <t>["isin-RU000A101MQ3", "isin-RU000A102Q90", "isin-RU000A102BC4", "isin-RU000A102770", "isin-RU000A102SL9", "isin-RU000A1036C0", "isin-RU000A103D60", "isin-RU000A101UM5", "isin-RU000A101ZK8", "isin-RU000A102374", "isin-RU000A103232", "isin-RU000A102YY0", "isin-RU000A101KR5", "isin-RU000A102FD3", "isin-RU000A103GZ2", "isin-RU000A103MY3", "isin-RU000A102MW9", "isin-RU000A101R74"]</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>["ru-inn-7743289272", "ru-inn-7701657100", "ru-inn-2308299972", "ru-inn-5244022664", "ru-inn-5904037892", "ru-inn-6320085325", "ru-inn-7702527954", "ru-inn-9728043461", "ru-inn-2531010480", "ru-inn-7704492383", "ru-inn-4101113738", "ru-inn-7725743542", "ru-inn-5507303700", "ru-inn-9704194045", "ru-inn-9714058147", "ru-inn-7733711248", "ru-inn-7701847158"]</t>
+          <t>["ru-inn-7743289272", "ru-inn-4101113738", "ru-inn-5507303700", "ru-inn-7704492383", "ru-inn-5904037892", "ru-inn-9728043461", "ru-inn-7733711248", "ru-inn-5244022664", "ru-inn-9714058147", "ru-inn-2531010480", "ru-inn-7701847158", "ru-inn-7702527954", "ru-inn-2308299972", "ru-inn-9704194045", "ru-inn-6320085325", "ru-inn-7701657100", "ru-inn-7725743542"]</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>["ua-edr-8bacf8ee166e0fc5abafd69917b524e0b3642103", "ua-edr-5a986e1ed9b47d8b57f62a4189e7a87517ed3438", "ua-edr-728dfe0fb5c472255c5d6676a3ee384785c5a62f", "ua-edr-99df79a495063e953965645e3c0bb34f312f40a2", "ua-edr-f1f7d80410597a4639345afefd450f4feab86fbc", "ua-edr-013090a414ba966e9b63fa324e4177ee0f20082b", "ua-edr-6002e691285c1f0f44c1bf301c1ac878cec8a859", "ua-edr-9556f1bc706781002b4a1c78759637b93b530596", "ua-edr-5e745987f6c7f714680d0b389c413b2df273ade3", "ua-edr-01627dafa2a14d4963b5d73f2a46624d71c97d7c", "ua-edr-ed93bcdb6a849d8ea9f0e733c2db19da3cf6eb52", "ua-edr-429ddf533e5221aafb2d27580255bf6d189480c3", "ua-edr-841cbcb837a32baffda0de1e59414a89a6bee339", "ua-edr-a74c66ffe91a9489158df4ec8f91b0d647d4e8ce", "ua-edr-abc9cafe239f1758d1800119763500502ed6acd7", "ua-edr-502c53beb1b493e2575fe161f8df265d6ce7eff4", "ua-edr-0877ee1e12f4cf3d331442fbb2ee500073e2f28c"]</t>
+          <t>["ua-edr-5e745987f6c7f714680d0b389c413b2df273ade3", "ua-edr-99df79a495063e953965645e3c0bb34f312f40a2", "ua-edr-013090a414ba966e9b63fa324e4177ee0f20082b", "ua-edr-9556f1bc706781002b4a1c78759637b93b530596", "ua-edr-429ddf533e5221aafb2d27580255bf6d189480c3", "ua-edr-6002e691285c1f0f44c1bf301c1ac878cec8a859", "ua-edr-8bacf8ee166e0fc5abafd69917b524e0b3642103", "ua-edr-728dfe0fb5c472255c5d6676a3ee384785c5a62f", "ua-edr-f1f7d80410597a4639345afefd450f4feab86fbc", "ua-edr-841cbcb837a32baffda0de1e59414a89a6bee339", "ua-edr-01627dafa2a14d4963b5d73f2a46624d71c97d7c", "ua-edr-502c53beb1b493e2575fe161f8df265d6ce7eff4", "ua-edr-abc9cafe239f1758d1800119763500502ed6acd7", "ua-edr-0877ee1e12f4cf3d331442fbb2ee500073e2f28c", "ua-edr-ed93bcdb6a849d8ea9f0e733c2db19da3cf6eb52", "ua-edr-5a986e1ed9b47d8b57f62a4189e7a87517ed3438", "ua-edr-a74c66ffe91a9489158df4ec8f91b0d647d4e8ce"]</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>["us-bis-export-03a3131d777c0b0575f941d28b30cfac7a0bfe61", "us-bis-export-4dde4d81c422e0f99b9683ca4eb18c2392155e66", "us-bis-export-36fad77b3c3b0ed0ab420e0c78ba583f2c97eaec", "us-bis-export-535f1b58120e7716fa25ed80b1456b67c4156473", "us-bis-export-9642b172a01249feb8ddeda82ac3d0d8b7b2bb90", "us-bis-export-f48912305c4dbcc6bb8632385fc391070974773d", "us-bis-export-995e9097a29d10642017db31ba22f09e344e297c", "us-bis-export-0f7514b15e893f05152ab60895ba05e2f04eab02", "us-bis-export-bb0c4774e8ff1b1b178c383784b9f07610e38caf", "us-bis-export-9e57b0d8a1e9d2f89cc79b48ca81dc9ca509521d", "us-bis-export-43bd1392fc4f3113c614c4c2b359c7adb2e31d79", "us-bis-export-41786fd0bd0a1322671f5091163b8bf2b12d149f", "us-bis-export-f59ed2b7aa0178d73365395b38ded03461840d95", "us-bis-export-634ad637ca4a0ae524073c800a55e83a6ca5b091", "us-bis-export-ce7306e097264749e060f167284409070209a2c1", "us-bis-export-257a072ab7741aac127bbc27219b9e586a81fafd", "us-bis-export-02a71f0a0b4df2ec61183537fd02e6a84266b4a4"]</t>
+          <t>["us-bis-export-bb0c4774e8ff1b1b178c383784b9f07610e38caf", "us-bis-export-9642b172a01249feb8ddeda82ac3d0d8b7b2bb90", "us-bis-export-9e57b0d8a1e9d2f89cc79b48ca81dc9ca509521d", "us-bis-export-4dde4d81c422e0f99b9683ca4eb18c2392155e66", "us-bis-export-03a3131d777c0b0575f941d28b30cfac7a0bfe61", "us-bis-export-995e9097a29d10642017db31ba22f09e344e297c", "us-bis-export-535f1b58120e7716fa25ed80b1456b67c4156473", "us-bis-export-ce7306e097264749e060f167284409070209a2c1", "us-bis-export-02a71f0a0b4df2ec61183537fd02e6a84266b4a4", "us-bis-export-41786fd0bd0a1322671f5091163b8bf2b12d149f", "us-bis-export-0f7514b15e893f05152ab60895ba05e2f04eab02", "us-bis-export-f48912305c4dbcc6bb8632385fc391070974773d", "us-bis-export-43bd1392fc4f3113c614c4c2b359c7adb2e31d79", "us-bis-export-f59ed2b7aa0178d73365395b38ded03461840d95", "us-bis-export-634ad637ca4a0ae524073c800a55e83a6ca5b091", "us-bis-export-36fad77b3c3b0ed0ab420e0c78ba583f2c97eaec", "us-bis-export-257a072ab7741aac127bbc27219b9e586a81fafd"]</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>["cy-ee56eb8c443a7615cb2b80aa785d7ede2b599cfa", "cy-afeba2ac035744cffb623f27a1152f76b0d0ebb7", "cy-4b132c7603b97c49a8b5b15b0da3106a1ea8d625", "cy-a23858f976cf121dbb0014dfb385cf0cdda413ac", "cy-4d7b8e3ab7f31d5fd7e8623938d54286dd429556", "cy-29970d3344c0d0b2d67019015b8475dce8c38478", "NK-VRJum2fRYwvTJRm9xRNg84", "cy-5b0538dfca5c3dfde24d94b4603942e73518c070", "cy-8389a85db6b70ffb8cb29d498a4d1e898ed069f5", "cy-223088d9245ddd2288b4990b254418c8ea8f1fce", "cy-d3ee69c8b3ea70a47c58ba36b4bd3c98f4ae6cbb", "cy-8dd3eb80d265f75dad9a9a3d1359b4ff7801951f", "cy-ce05129da07e72c76a8d06820102b17ba60f9341", "cy-79e79a017d1016b1e668e727688b1c9bfbe95854", "cy-f3b61a663b6de3cdc27b53e99e9c15b21d12961a", "cy-d802e23b9fcbaacf8705ddde7a23cf0c447cf866"]</t>
+          <t>["cy-8dd3eb80d265f75dad9a9a3d1359b4ff7801951f", "NK-VRJum2fRYwvTJRm9xRNg84", "cy-d802e23b9fcbaacf8705ddde7a23cf0c447cf866", "cy-29970d3344c0d0b2d67019015b8475dce8c38478", "cy-ee56eb8c443a7615cb2b80aa785d7ede2b599cfa", "cy-79e79a017d1016b1e668e727688b1c9bfbe95854", "cy-4b132c7603b97c49a8b5b15b0da3106a1ea8d625", "cy-f3b61a663b6de3cdc27b53e99e9c15b21d12961a", "cy-a23858f976cf121dbb0014dfb385cf0cdda413ac", "cy-223088d9245ddd2288b4990b254418c8ea8f1fce", "cy-5b0538dfca5c3dfde24d94b4603942e73518c070", "cy-afeba2ac035744cffb623f27a1152f76b0d0ebb7", "cy-d3ee69c8b3ea70a47c58ba36b4bd3c98f4ae6cbb", "cy-4d7b8e3ab7f31d5fd7e8623938d54286dd429556", "cy-ce05129da07e72c76a8d06820102b17ba60f9341", "cy-8389a85db6b70ffb8cb29d498a4d1e898ed069f5"]</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>["pk-cnic-3320371645081", "pk-cnic-5340256608773", "pk-cnic-3310280324005", "pk-cnic-5550103456497", "pk-cnic-3240271987885", "pk-cnic-3840359820147", "pk-cnic-4230138896977", "pk-cnic-3540116384153", "pk-cnic-3240413956031", "pk-cnic-3320267483611", "pk-cnic-3840177568133", "Q109767291", "Q85739406", "pk-cnic-3120570621759", "pk-cnic-3840320506127", "pk-cnic-5630110723091"]</t>
+          <t>["Q109767291", "pk-cnic-3240413956031", "Q85739406", "pk-cnic-3240271987885", "pk-cnic-5630110723091", "pk-cnic-3120570621759", "pk-cnic-4230138896977", "pk-cnic-3540116384153", "pk-cnic-3840320506127", "pk-cnic-3840359820147", "pk-cnic-3320267483611", "pk-cnic-5340256608773", "pk-cnic-3840177568133", "pk-cnic-5550103456497", "pk-cnic-3310280324005", "pk-cnic-3320371645081"]</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>["isin-RU000A10ASD4", "isin-RU000A10B3Y6", "isin-RU000A10BT00", "isin-RU000A10A026", "isin-RU000A108ZU2", "isin-RU000A109890", "isin-RU000A10CRB6", "isin-RU000A10D3S6", "isin-RU000A10BVF1", "isin-RU000A10BBE6", "isin-RU000A10C3M0", "isin-RU000A109B82", "isin-RU000A10B4X6", "isin-RU000A10C5Z7", "isin-RU000A10BY52", "isin-RU000A10BNK8"]</t>
+          <t>["isin-RU000A109890", "isin-RU000A108ZU2", "isin-RU000A10B4X6", "isin-RU000A10BT00", "isin-RU000A10BY52", "isin-RU000A10B3Y6", "isin-RU000A10BBE6", "isin-RU000A10CRB6", "isin-RU000A10C3M0", "isin-RU000A10ASD4", "isin-RU000A10D3S6", "isin-RU000A10A026", "isin-RU000A10BNK8", "isin-RU000A10BVF1", "isin-RU000A109B82", "isin-RU000A10C5Z7"]</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>["ru-inn-7716873898", "ru-inn-4307020290", "ru-inn-5643022352", "ru-inn-7705555702", "ru-inn-3849037461", "ru-inn-9108122988", "ru-inn-3311024680", "ru-inn-9718180638", "ru-inn-1800001982", "ru-inn-5047263660", "ru-inn-7714966755", "ru-inn-9701171900", "ru-inn-5044047196", "ru-inn-9731150128", "ru-inn-5260478292", "ru-inn-7448136590"]</t>
+          <t>["ru-inn-9731150128", "ru-inn-9718180638", "ru-inn-3311024680", "ru-inn-5047263660", "ru-inn-5643022352", "ru-inn-9108122988", "ru-inn-7716873898", "ru-inn-3849037461", "ru-inn-4307020290", "ru-inn-5260478292", "ru-inn-7714966755", "ru-inn-9701171900", "ru-inn-7448136590", "ru-inn-1800001982", "ru-inn-5044047196", "ru-inn-7705555702"]</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>["ru-inn-5048018929", "ru-inn-4205327082", "ru-inn-7841098406", "ru-inn-9714059359", "ru-inn-7805250052", "ru-inn-4826127992", "ru-inn-7707430353", "ru-inn-7725371453", "ru-inn-4252000920", "ru-inn-7713495327", "ru-inn-9731069244", "ru-inn-9715422085", "ru-inn-9729006751", "ru-inn-5257125360", "ru-inn-5038111005", "ru-inn-2221222189"]</t>
+          <t>["ru-inn-9729006751", "ru-inn-9715422085", "ru-inn-7841098406", "ru-inn-7707430353", "ru-inn-4826127992", "ru-inn-7713495327", "ru-inn-7725371453", "ru-inn-5257125360", "ru-inn-9714059359", "ru-inn-9731069244", "ru-inn-7805250052", "ru-inn-5048018929", "ru-inn-2221222189", "ru-inn-4205327082", "ru-inn-4252000920", "ru-inn-5038111005"]</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -1730,7 +1730,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>["ua-edr-9472168f49fb20e1f1753e691baa240e224265c9", "ua-edr-5d094c3ddabaa0437cd1b69ecc5b488bf77d38f0", "ua-edr-d86dbb88879c1599e78c6f5e787730bed6e32aa4", "ua-edr-3ea3da70f834441deb8f77c450f28457bc1e8b1a", "ua-edr-cede6ceb18599f5f73914e1f4ed83e42dfca5342", "ua-edr-c6d42d5b4e212aafc7207f7557f33b4654e4917c", "ua-edr-5af61c1a7efbccf8ae56504a447d8d84f1fd4dea", "ua-edr-82b0c874b4a03e4409d92323cdf16f13a4cb3cd4", "ua-edr-4e1a6057dbb02f9a0b2cc6ceb3871b87ef2fd53c", "ua-edr-5e5ca2182dd3bcf0956a2d6c4e86a9f797dd4ba0", "ua-edr-4242168f1602d66b7396365d8a2962f379c89686", "ua-edr-5483750ea8a6040702cf8e6ee08911e13984cc18", "ua-edr-ca1159568f1d4eec560aed6a9a5bae8d46dcba28", "ua-edr-22154614206aa9662c46f509ce04b1103dd9a297", "ua-edr-a5acd52925972aadcda603231fafc1282f41a1fe", "ua-edr-e9b1aa90d0ad3e259df32472efe032ad4841b391"]</t>
+          <t>["ua-edr-5d094c3ddabaa0437cd1b69ecc5b488bf77d38f0", "ua-edr-22154614206aa9662c46f509ce04b1103dd9a297", "ua-edr-5e5ca2182dd3bcf0956a2d6c4e86a9f797dd4ba0", "ua-edr-cede6ceb18599f5f73914e1f4ed83e42dfca5342", "ua-edr-5af61c1a7efbccf8ae56504a447d8d84f1fd4dea", "ua-edr-4e1a6057dbb02f9a0b2cc6ceb3871b87ef2fd53c", "ua-edr-c6d42d5b4e212aafc7207f7557f33b4654e4917c", "ua-edr-82b0c874b4a03e4409d92323cdf16f13a4cb3cd4", "ua-edr-e9b1aa90d0ad3e259df32472efe032ad4841b391", "ua-edr-d86dbb88879c1599e78c6f5e787730bed6e32aa4", "ua-edr-3ea3da70f834441deb8f77c450f28457bc1e8b1a", "ua-edr-4242168f1602d66b7396365d8a2962f379c89686", "ua-edr-9472168f49fb20e1f1753e691baa240e224265c9", "ua-edr-ca1159568f1d4eec560aed6a9a5bae8d46dcba28", "ua-edr-a5acd52925972aadcda603231fafc1282f41a1fe", "ua-edr-5483750ea8a6040702cf8e6ee08911e13984cc18"]</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>["cy-c96782983263f75ffc723af2968a68b4b0e0bd45", "cy-d9a18fb5f8d757145ea4131c7a5446fbfe9e0e6b", "cy-8a07910d7dd5f25ee391fe6e2640dd67454b6d2e", "cy-00a9ff29cf59b91407a36a8fcb3274cae24a2312", "cy-2a20390a8c6760c606be6c7f8dabf1785bab8c51", "cy-65dd5c869dc51903bfd595c75216fb000a2f0f00", "cy-19a1e020d6e925c3c8c5e44d9636d3d84629f7ec", "cy-bfbe84015d82dc0477b23fe768a0e10ec220bffb", "cy-e87a101b317b996481ffb57f03fe3597bfc80765", "cy-f149aa3addc53ce34e9108c136605044a1fc898e", "cy-5d37aafc2f4a74217ce0f096b9e3ee6442ee3754", "cy-b0ec6aadac28597e7bcc503cd1b9a1115cedf151", "cy-90e2bb1252c2a89cdd2457ec8bf867907305005a", "cy-2e3e9e6cbc6b8a74eaa0d009cf4f99e27ef9fd8b", "cy-0d1a41bbad9a884592094a643c65691b5c50b6a5"]</t>
+          <t>["cy-8a07910d7dd5f25ee391fe6e2640dd67454b6d2e", "cy-bfbe84015d82dc0477b23fe768a0e10ec220bffb", "cy-0d1a41bbad9a884592094a643c65691b5c50b6a5", "cy-65dd5c869dc51903bfd595c75216fb000a2f0f00", "cy-c96782983263f75ffc723af2968a68b4b0e0bd45", "cy-2e3e9e6cbc6b8a74eaa0d009cf4f99e27ef9fd8b", "cy-5d37aafc2f4a74217ce0f096b9e3ee6442ee3754", "cy-19a1e020d6e925c3c8c5e44d9636d3d84629f7ec", "cy-d9a18fb5f8d757145ea4131c7a5446fbfe9e0e6b", "cy-e87a101b317b996481ffb57f03fe3597bfc80765", "cy-00a9ff29cf59b91407a36a8fcb3274cae24a2312", "cy-90e2bb1252c2a89cdd2457ec8bf867907305005a", "cy-b0ec6aadac28597e7bcc503cd1b9a1115cedf151", "cy-f149aa3addc53ce34e9108c136605044a1fc898e", "cy-2a20390a8c6760c606be6c7f8dabf1785bab8c51"]</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>

</xml_diff>